<commit_message>
feat(kam): update verified partners workbook with merged Fresh, Agat, and Dobrolyubova transfers
</commit_message>
<xml_diff>
--- a/Закрепление_партнеров_по_КАМ_Сентябрь_2026.xlsx
+++ b/Закрепление_партнеров_по_КАМ_Сентябрь_2026.xlsx
@@ -15,9 +15,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Валерия Солдатова" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Андрей Кузнецов'!$A$4:$J$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Андрей Кузнецов'!$A$4:$J$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Алексей Чихарев'!$A$4:$J$214</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Евгения Добролюбова'!$A$4:$J$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Евгения Добролюбова'!$A$4:$J$100</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Светлана Дариенко'!$A$4:$J$128</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Валерия Солдатова'!$A$4:$J$215</definedName>
   </definedNames>
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>196</v>
@@ -667,16 +667,16 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
@@ -697,13 +697,13 @@
         <v>124</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E8" s="10" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="D10" s="14" t="n">
         <v>771</v>
@@ -770,7 +770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -778,7 +778,7 @@
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
@@ -795,7 +795,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Всего объектов в портфеле: 72 ДЦ. Источник: OEM СберАвто финал (15)</t>
+          <t>Всего объектов в портфеле: 69 ДЦ. Источник: OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -2334,13 +2334,13 @@
         </is>
       </c>
       <c r="G38" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H38" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I38" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J38" s="17" t="inlineStr">
         <is>
@@ -2378,13 +2378,13 @@
         </is>
       </c>
       <c r="G39" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H39" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I39" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J39" s="17" t="inlineStr">
         <is>
@@ -2422,13 +2422,13 @@
         </is>
       </c>
       <c r="G40" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H40" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I40" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J40" s="17" t="inlineStr">
         <is>
@@ -2466,13 +2466,13 @@
         </is>
       </c>
       <c r="G41" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H41" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I41" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J41" s="17" t="inlineStr">
         <is>
@@ -2506,13 +2506,13 @@
         </is>
       </c>
       <c r="G42" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H42" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I42" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J42" s="17" t="inlineStr">
         <is>
@@ -2546,13 +2546,13 @@
         </is>
       </c>
       <c r="G43" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H43" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I43" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J43" s="17" t="inlineStr">
         <is>
@@ -2590,13 +2590,13 @@
         </is>
       </c>
       <c r="G44" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H44" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I44" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J44" s="17" t="inlineStr">
         <is>
@@ -2634,13 +2634,13 @@
         </is>
       </c>
       <c r="G45" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H45" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I45" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J45" s="17" t="inlineStr">
         <is>
@@ -2678,13 +2678,13 @@
         </is>
       </c>
       <c r="G46" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H46" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I46" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J46" s="17" t="inlineStr">
         <is>
@@ -2722,13 +2722,13 @@
         </is>
       </c>
       <c r="G47" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H47" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I47" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J47" s="17" t="inlineStr">
         <is>
@@ -2766,13 +2766,13 @@
         </is>
       </c>
       <c r="G48" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H48" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I48" s="18" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J48" s="17" t="inlineStr">
         <is>
@@ -3393,42 +3393,46 @@
       </c>
     </row>
     <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="16" t="n">
+      <c r="A63" s="4" t="n">
         <v>59</v>
       </c>
-      <c r="B63" s="17" t="inlineStr">
-        <is>
-          <t>АГАТ ООО "АКЦЕНТ</t>
-        </is>
-      </c>
-      <c r="C63" s="17" t="inlineStr">
-        <is>
-          <t>АГАТ ООО "АКЦЕНТ" ONLINE</t>
-        </is>
-      </c>
-      <c r="D63" s="16" t="inlineStr"/>
-      <c r="E63" s="17" t="inlineStr">
-        <is>
-          <t>РФ</t>
-        </is>
-      </c>
-      <c r="F63" s="17" t="inlineStr">
-        <is>
-          <t>JETOUR</t>
-        </is>
-      </c>
-      <c r="G63" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="H63" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I63" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="J63" s="17" t="inlineStr">
-        <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Fresh Haval мин воды</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Fresh Haval мин воды</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>3443137377</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Минеральные Воды</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>HAVAL</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" s="7" t="inlineStr">
+        <is>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -3438,23 +3442,27 @@
       </c>
       <c r="B64" s="11" t="inlineStr">
         <is>
-          <t>CHERY Фреш</t>
+          <t>Fresh Haval Ростов</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>СберАвто</t>
-        </is>
-      </c>
-      <c r="D64" s="8" t="inlineStr"/>
+          <t>Fresh Haval Ростов</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>3443137377</t>
+        </is>
+      </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Ростов-на-Дону</t>
         </is>
       </c>
       <c r="F64" s="11" t="inlineStr">
         <is>
-          <t>CHERY &amp; TENET</t>
+          <t>HAVAL</t>
         </is>
       </c>
       <c r="G64" s="10" t="n">
@@ -3468,7 +3476,7 @@
       </c>
       <c r="J64" s="11" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -3478,27 +3486,23 @@
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Fresh Haval мин воды</t>
+          <t>Team63Auto</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>Fresh Haval мин воды</t>
-        </is>
-      </c>
-      <c r="D65" s="4" t="inlineStr">
-        <is>
-          <t>3443137377</t>
-        </is>
-      </c>
+          <t>СберАвто, Team63Auto</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr"/>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>Минеральные Воды</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>HAVAL</t>
+          <t>HYUNDAI, CHERY &amp; TENET</t>
         </is>
       </c>
       <c r="G65" s="6" t="n">
@@ -3512,7 +3516,7 @@
       </c>
       <c r="J65" s="7" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -3522,27 +3526,27 @@
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>Fresh Haval Ростов</t>
+          <t>Tenet Центр Ника Авто</t>
         </is>
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>Fresh Haval Ростов</t>
+          <t>Tenet Центр Ника Авто</t>
         </is>
       </c>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>3443137377</t>
+          <t>5638074027</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
         <is>
-          <t>Ростов-на-Дону</t>
+          <t>Орск</t>
         </is>
       </c>
       <c r="F66" s="11" t="inlineStr">
         <is>
-          <t>HAVAL</t>
+          <t>CHERY</t>
         </is>
       </c>
       <c r="G66" s="10" t="n">
@@ -3566,23 +3570,27 @@
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Team63Auto</t>
+          <t>ГК Арконт</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>Team63Auto, СберАвто</t>
-        </is>
-      </c>
-      <c r="D67" s="4" t="inlineStr"/>
+          <t>ГК Арконт</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>3443113810</t>
+        </is>
+      </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Волгоград</t>
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>HYUNDAI, CHERY &amp; TENET</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G67" s="6" t="n">
@@ -3596,7 +3604,7 @@
       </c>
       <c r="J67" s="7" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -3606,22 +3614,22 @@
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
-          <t>Tenet Центр Ника Авто</t>
+          <t>ТВС Моторс</t>
         </is>
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>Tenet Центр Ника Авто</t>
+          <t>ТВС Моторс</t>
         </is>
       </c>
       <c r="D68" s="8" t="inlineStr">
         <is>
-          <t>5638074027</t>
+          <t>5610215334</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>Орск</t>
+          <t>Оренбург</t>
         </is>
       </c>
       <c r="F68" s="11" t="inlineStr">
@@ -3650,27 +3658,27 @@
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>ГК Арконт</t>
+          <t>Фрэш Авто</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>ГК Арконт</t>
+          <t>Фрэш Авто</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>3443113810</t>
+          <t>7724423589</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>Волгоград</t>
+          <t>Воронеж</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>CHERY</t>
         </is>
       </c>
       <c r="G69" s="6" t="n">
@@ -3694,23 +3702,27 @@
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>Приоритет_Fresh</t>
+          <t>Чери Центр Автофорум</t>
         </is>
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>Приоритет_Fresh</t>
-        </is>
-      </c>
-      <c r="D70" s="8" t="inlineStr"/>
+          <t>Чери Центр Автофорум</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>6452947574</t>
+        </is>
+      </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Саратов</t>
         </is>
       </c>
       <c r="F70" s="11" t="inlineStr">
         <is>
-          <t>MERCEDES, NISSAN, LEXUS</t>
+          <t>CHERY</t>
         </is>
       </c>
       <c r="G70" s="10" t="n">
@@ -3724,7 +3736,7 @@
       </c>
       <c r="J70" s="11" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -3734,22 +3746,22 @@
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>ТВС Моторс</t>
+          <t>ЧЕРИ ЦЕНТР АГАТ-АВТО Онлайн Иркутск</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>ТВС Моторс</t>
+          <t>ЧЕРИ ЦЕНТР АГАТ-АВТО Онлайн Иркутск</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>5610215334</t>
+          <t>3804048079</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>Оренбург</t>
+          <t>Иркутск</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr">
@@ -3778,22 +3790,22 @@
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>Фрэш Авто</t>
+          <t>ЧЕРИ ЦЕНТР НИЖЕГОРОДЕЦ ОНЛАЙН</t>
         </is>
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>Фрэш Авто</t>
+          <t>ЧЕРИ ЦЕНТР НИЖЕГОРОДЕЦ ОНЛАЙН</t>
         </is>
       </c>
       <c r="D72" s="8" t="inlineStr">
         <is>
-          <t>7724423589</t>
+          <t>5257164835</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>Воронеж</t>
+          <t>Нижний Новгород</t>
         </is>
       </c>
       <c r="F72" s="11" t="inlineStr">
@@ -3822,22 +3834,22 @@
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>Чери Центр Автофорум</t>
+          <t>ЧЕРИ ЦЕНТР ПЛАНЕТА АВТО ВОСТОК</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>Чери Центр Автофорум</t>
+          <t>ЧЕРИ ЦЕНТР ПЛАНЕТА АВТО ВОСТОК</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>6452947574</t>
+          <t>7447124619</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>Саратов</t>
+          <t>Челябинск</t>
         </is>
       </c>
       <c r="F73" s="7" t="inlineStr">
@@ -3860,169 +3872,37 @@
         </is>
       </c>
     </row>
-    <row r="74" ht="20" customHeight="1">
-      <c r="A74" s="8" t="n">
-        <v>70</v>
-      </c>
-      <c r="B74" s="11" t="inlineStr">
-        <is>
-          <t>ЧЕРИ ЦЕНТР АГАТ-АВТО Онлайн Иркутск</t>
-        </is>
-      </c>
-      <c r="C74" s="11" t="inlineStr">
-        <is>
-          <t>ЧЕРИ ЦЕНТР АГАТ-АВТО Онлайн Иркутск</t>
-        </is>
-      </c>
-      <c r="D74" s="8" t="inlineStr">
-        <is>
-          <t>3804048079</t>
-        </is>
-      </c>
-      <c r="E74" s="11" t="inlineStr">
-        <is>
-          <t>Иркутск</t>
-        </is>
-      </c>
-      <c r="F74" s="11" t="inlineStr">
-        <is>
-          <t>CHERY</t>
-        </is>
-      </c>
-      <c r="G74" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H74" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I74" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J74" s="11" t="inlineStr">
-        <is>
-          <t>OEM СберАвто финал (15)</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="A75" s="4" t="n">
-        <v>71</v>
-      </c>
-      <c r="B75" s="7" t="inlineStr">
-        <is>
-          <t>ЧЕРИ ЦЕНТР НИЖЕГОРОДЕЦ ОНЛАЙН</t>
-        </is>
-      </c>
-      <c r="C75" s="7" t="inlineStr">
-        <is>
-          <t>ЧЕРИ ЦЕНТР НИЖЕГОРОДЕЦ ОНЛАЙН</t>
-        </is>
-      </c>
-      <c r="D75" s="4" t="inlineStr">
-        <is>
-          <t>5257164835</t>
-        </is>
-      </c>
-      <c r="E75" s="7" t="inlineStr">
-        <is>
-          <t>Нижний Новгород</t>
-        </is>
-      </c>
-      <c r="F75" s="7" t="inlineStr">
-        <is>
-          <t>CHERY</t>
-        </is>
-      </c>
-      <c r="G75" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H75" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I75" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J75" s="7" t="inlineStr">
-        <is>
-          <t>OEM СберАвто финал (15)</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="20" customHeight="1">
-      <c r="A76" s="8" t="n">
-        <v>72</v>
-      </c>
-      <c r="B76" s="11" t="inlineStr">
-        <is>
-          <t>ЧЕРИ ЦЕНТР ПЛАНЕТА АВТО ВОСТОК</t>
-        </is>
-      </c>
-      <c r="C76" s="11" t="inlineStr">
-        <is>
-          <t>ЧЕРИ ЦЕНТР ПЛАНЕТА АВТО ВОСТОК</t>
-        </is>
-      </c>
-      <c r="D76" s="8" t="inlineStr">
-        <is>
-          <t>7447124619</t>
-        </is>
-      </c>
-      <c r="E76" s="11" t="inlineStr">
-        <is>
-          <t>Челябинск</t>
-        </is>
-      </c>
-      <c r="F76" s="11" t="inlineStr">
-        <is>
-          <t>CHERY</t>
-        </is>
-      </c>
-      <c r="G76" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H76" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I76" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J76" s="11" t="inlineStr">
-        <is>
-          <t>OEM СберАвто финал (15)</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="24" customHeight="1">
-      <c r="A77" s="12" t="inlineStr"/>
-      <c r="B77" s="13" t="inlineStr">
+    <row r="74" ht="24" customHeight="1">
+      <c r="A74" s="12" t="inlineStr"/>
+      <c r="B74" s="13" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="C77" s="13" t="inlineStr">
-        <is>
-          <t>72 объектов</t>
-        </is>
-      </c>
-      <c r="D77" s="12" t="n"/>
-      <c r="E77" s="12" t="n"/>
-      <c r="F77" s="12" t="n"/>
-      <c r="G77" s="14">
-        <f>SUM(G5:G76)</f>
+      <c r="C74" s="13" t="inlineStr">
+        <is>
+          <t>69 объектов</t>
+        </is>
+      </c>
+      <c r="D74" s="12" t="n"/>
+      <c r="E74" s="12" t="n"/>
+      <c r="F74" s="12" t="n"/>
+      <c r="G74" s="14">
+        <f>SUM(G5:G73)</f>
         <v/>
       </c>
-      <c r="H77" s="14">
-        <f>SUM(H5:H76)</f>
+      <c r="H74" s="14">
+        <f>SUM(H5:H73)</f>
         <v/>
       </c>
-      <c r="I77" s="14">
-        <f>SUM(I5:I76)</f>
+      <c r="I74" s="14">
+        <f>SUM(I5:I73)</f>
         <v/>
       </c>
-      <c r="J77" s="12" t="n"/>
+      <c r="J74" s="12" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J76"/>
+  <autoFilter ref="A4:J73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6934,7 +6814,7 @@
       </c>
       <c r="C69" s="17" t="inlineStr">
         <is>
-          <t>Online ЭКСПЕРТ АВТО ОРЕНБУРГ, ООО "ЭКСПЕРТ СВ ОРЕНБУРГ" Online</t>
+          <t>ООО "ЭКСПЕРТ СВ ОРЕНБУРГ" Online, Online ЭКСПЕРТ АВТО ОРЕНБУРГ</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr"/>
@@ -6945,7 +6825,7 @@
       </c>
       <c r="F69" s="17" t="inlineStr">
         <is>
-          <t>HAVAL, GAC, LADA</t>
+          <t>LADA, GAC, HAVAL</t>
         </is>
       </c>
       <c r="G69" s="18" t="n">
@@ -7634,7 +7514,7 @@
       </c>
       <c r="C85" s="17" t="inlineStr">
         <is>
-          <t>ГК Техцентр Гранд, ООО "МЛАДА - АВТО" online</t>
+          <t>ООО "МЛАДА - АВТО" online, ГК Техцентр Гранд</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr"/>
@@ -10730,7 +10610,7 @@
       </c>
       <c r="C156" s="17" t="inlineStr">
         <is>
-          <t>Online ООО АВТО-МОТОРС Лада, ONLINE ФДЦ АВТО-МОТОРС Сургут</t>
+          <t>ONLINE ФДЦ АВТО-МОТОРС Сургут, Online ООО АВТО-МОТОРС Лада</t>
         </is>
       </c>
       <c r="D156" s="16" t="inlineStr"/>
@@ -10781,7 +10661,7 @@
       </c>
       <c r="F157" s="7" t="inlineStr">
         <is>
-          <t>JETOUR, Belgee, NISSAN</t>
+          <t>JETOUR, RENAULT, EXEED</t>
         </is>
       </c>
       <c r="G157" s="6" t="n">
@@ -13324,7 +13204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J100"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -13349,7 +13229,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Всего объектов в портфеле: 95 ДЦ. Источник: OEM СберАвто финал (15)</t>
+          <t>Всего объектов в портфеле: 96 ДЦ. Источник: OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -14241,7 +14121,7 @@
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>ООО "МБ-БРЯНСК" ONLINE, ГК БН-МОТОРС, БНМ</t>
+          <t>ГК БН-МОТОРС, БНМ, ООО "МБ-БРЯНСК" ONLINE</t>
         </is>
       </c>
       <c r="D24" s="16" t="inlineStr"/>
@@ -14252,7 +14132,7 @@
       </c>
       <c r="F24" s="17" t="inlineStr">
         <is>
-          <t>SOUEAST, LADA, JETOUR</t>
+          <t>LADA, SOUEAST, JETOUR</t>
         </is>
       </c>
       <c r="G24" s="18" t="n">
@@ -14456,7 +14336,7 @@
       </c>
       <c r="F29" s="17" t="inlineStr">
         <is>
-          <t>OMODA &amp; JAECOO, CHERY &amp; TENET</t>
+          <t>CHERY &amp; TENET, OMODA &amp; JAECOO</t>
         </is>
       </c>
       <c r="G29" s="18" t="n">
@@ -14617,7 +14497,7 @@
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
-          <t>ONLINE Олимп, ONLINE Олимп (ООО "ТЕМП АВТО КУБАНЬ")</t>
+          <t>ONLINE Олимп (ООО "ТЕМП АВТО КУБАНЬ"), ONLINE Олимп</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr"/>
@@ -14657,7 +14537,7 @@
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>ONLINE ООО "АВТОБАН-ВОСТОК", Приоритет_Автобан</t>
+          <t>Приоритет_Автобан, ONLINE ООО "АВТОБАН-ВОСТОК"</t>
         </is>
       </c>
       <c r="D34" s="16" t="inlineStr"/>
@@ -14668,7 +14548,7 @@
       </c>
       <c r="F34" s="17" t="inlineStr">
         <is>
-          <t>SOUEAST, SKODA, JETOUR</t>
+          <t>SKODA, SOUEAST, JETOUR</t>
         </is>
       </c>
       <c r="G34" s="18" t="n">
@@ -14948,27 +14828,23 @@
       </c>
       <c r="B41" s="17" t="inlineStr">
         <is>
-          <t>ГК Сатурн 2</t>
+          <t>Авторитейл Диаманд</t>
         </is>
       </c>
       <c r="C41" s="17" t="inlineStr">
         <is>
-          <t>Сатурн 2</t>
-        </is>
-      </c>
-      <c r="D41" s="16" t="inlineStr">
-        <is>
-          <t>7449019666</t>
-        </is>
-      </c>
+          <t>Online ООО АВТО РИТЕЙЛ ДИАМАНТ / ГК Форвард</t>
+        </is>
+      </c>
+      <c r="D41" s="16" t="inlineStr"/>
       <c r="E41" s="17" t="inlineStr">
         <is>
-          <t>Челябинск</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F41" s="17" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>CHERY &amp; TENET</t>
         </is>
       </c>
       <c r="G41" s="18" t="n">
@@ -14982,7 +14858,7 @@
       </c>
       <c r="J41" s="17" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -15002,7 +14878,7 @@
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>5024106566</t>
+          <t>7449019666</t>
         </is>
       </c>
       <c r="E42" s="17" t="inlineStr">
@@ -15041,12 +14917,12 @@
       </c>
       <c r="C43" s="17" t="inlineStr">
         <is>
-          <t>Сатурн-2</t>
+          <t>Сатурн 2</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>7449019666</t>
+          <t>5024106566</t>
         </is>
       </c>
       <c r="E43" s="17" t="inlineStr">
@@ -15056,7 +14932,7 @@
       </c>
       <c r="F43" s="17" t="inlineStr">
         <is>
-          <t>CHANGAN</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G43" s="18" t="n">
@@ -15080,23 +14956,27 @@
       </c>
       <c r="B44" s="17" t="inlineStr">
         <is>
-          <t>Дебрянск Авто (Дебрянск Авто)</t>
+          <t>ГК Сатурн 2</t>
         </is>
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
-          <t>ООО "МБ-БРЯНСК" ONLINE</t>
-        </is>
-      </c>
-      <c r="D44" s="16" t="inlineStr"/>
+          <t>Сатурн-2</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>7449019666</t>
+        </is>
+      </c>
       <c r="E44" s="17" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Челябинск</t>
         </is>
       </c>
       <c r="F44" s="17" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>CHANGAN</t>
         </is>
       </c>
       <c r="G44" s="18" t="n">
@@ -15110,7 +14990,7 @@
       </c>
       <c r="J44" s="17" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -15120,22 +15000,18 @@
       </c>
       <c r="B45" s="17" t="inlineStr">
         <is>
-          <t>Леон Авто</t>
+          <t>Дебрянск Авто (Дебрянск Авто)</t>
         </is>
       </c>
       <c r="C45" s="17" t="inlineStr">
         <is>
-          <t>Леон Авто</t>
-        </is>
-      </c>
-      <c r="D45" s="16" t="inlineStr">
-        <is>
-          <t>1207901941</t>
-        </is>
-      </c>
+          <t>ООО "МБ-БРЯНСК" ONLINE</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr"/>
       <c r="E45" s="17" t="inlineStr">
         <is>
-          <t>Йошкар-Ола</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F45" s="17" t="inlineStr">
@@ -15154,7 +15030,7 @@
       </c>
       <c r="J45" s="17" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -15164,22 +15040,22 @@
       </c>
       <c r="B46" s="17" t="inlineStr">
         <is>
-          <t>ООО "АМР</t>
+          <t>Леон Авто</t>
         </is>
       </c>
       <c r="C46" s="17" t="inlineStr">
         <is>
-          <t>АМР</t>
+          <t>Леон Авто</t>
         </is>
       </c>
       <c r="D46" s="16" t="inlineStr">
         <is>
-          <t>9723110523</t>
+          <t>1207901941</t>
         </is>
       </c>
       <c r="E46" s="17" t="inlineStr">
         <is>
-          <t>Саратов</t>
+          <t>Йошкар-Ола</t>
         </is>
       </c>
       <c r="F46" s="17" t="inlineStr">
@@ -15208,27 +15084,27 @@
       </c>
       <c r="B47" s="17" t="inlineStr">
         <is>
-          <t>ООО "ВИП АВТО САМАРА</t>
+          <t>ООО "АМР</t>
         </is>
       </c>
       <c r="C47" s="17" t="inlineStr">
         <is>
-          <t>ВИП АВТО САМАРА</t>
+          <t>АМР</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>6312214182</t>
+          <t>9723110523</t>
         </is>
       </c>
       <c r="E47" s="17" t="inlineStr">
         <is>
-          <t>Самара</t>
+          <t>Саратов</t>
         </is>
       </c>
       <c r="F47" s="17" t="inlineStr">
         <is>
-          <t>OMODA</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G47" s="18" t="n">
@@ -15252,23 +15128,27 @@
       </c>
       <c r="B48" s="17" t="inlineStr">
         <is>
-          <t>ООО "ГЛАЗУРИТ</t>
+          <t>ООО "ВИП АВТО САМАРА</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>ООО "ГЛАЗУРИТ" online, ООО " ОК-ТРАНС " ONLINE</t>
-        </is>
-      </c>
-      <c r="D48" s="16" t="inlineStr"/>
+          <t>ВИП АВТО САМАРА</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr">
+        <is>
+          <t>6312214182</t>
+        </is>
+      </c>
       <c r="E48" s="17" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Самара</t>
         </is>
       </c>
       <c r="F48" s="17" t="inlineStr">
         <is>
-          <t>SOUEAST</t>
+          <t>OMODA</t>
         </is>
       </c>
       <c r="G48" s="18" t="n">
@@ -15282,7 +15162,7 @@
       </c>
       <c r="J48" s="17" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -15292,12 +15172,12 @@
       </c>
       <c r="B49" s="17" t="inlineStr">
         <is>
-          <t>ООО "САВ" - online</t>
+          <t>ООО "ГЛАЗУРИТ</t>
         </is>
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>ООО "САВ" - online</t>
+          <t>ООО "ГЛАЗУРИТ" online, ООО " ОК-ТРАНС " ONLINE</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr"/>
@@ -15332,12 +15212,12 @@
       </c>
       <c r="B50" s="17" t="inlineStr">
         <is>
-          <t>Самара-Лада</t>
+          <t>ООО "САВ" - online</t>
         </is>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>Самара-Лада (ООО Самара-Лада)/ Продажи МегаМаркета + Online, ONLINE Самара-Лада</t>
+          <t>ООО "САВ" - online</t>
         </is>
       </c>
       <c r="D50" s="16" t="inlineStr"/>
@@ -15348,7 +15228,7 @@
       </c>
       <c r="F50" s="17" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>SOUEAST</t>
         </is>
       </c>
       <c r="G50" s="18" t="n">
@@ -15372,22 +15252,18 @@
       </c>
       <c r="B51" s="17" t="inlineStr">
         <is>
-          <t>Сатурн-Р</t>
+          <t>Самара-Лада</t>
         </is>
       </c>
       <c r="C51" s="17" t="inlineStr">
         <is>
-          <t>Сатурн-Р</t>
-        </is>
-      </c>
-      <c r="D51" s="16" t="inlineStr">
-        <is>
-          <t>4501110065</t>
-        </is>
-      </c>
+          <t>ONLINE Самара-Лада, Самара-Лада (ООО Самара-Лада)/ Продажи МегаМаркета + Online</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="inlineStr"/>
       <c r="E51" s="17" t="inlineStr">
         <is>
-          <t>Пермь</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F51" s="17" t="inlineStr">
@@ -15406,7 +15282,7 @@
       </c>
       <c r="J51" s="17" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -15416,18 +15292,22 @@
       </c>
       <c r="B52" s="17" t="inlineStr">
         <is>
-          <t>Форвард Авто Лада Ижевск</t>
+          <t>Сатурн-Р</t>
         </is>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
-          <t>ONLINE ФОРВАРД Авто Ижевск (ООО "ФОРВАРД-АВТО")</t>
-        </is>
-      </c>
-      <c r="D52" s="16" t="inlineStr"/>
+          <t>Сатурн-Р</t>
+        </is>
+      </c>
+      <c r="D52" s="16" t="inlineStr">
+        <is>
+          <t>4501110065</t>
+        </is>
+      </c>
       <c r="E52" s="17" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Пермь</t>
         </is>
       </c>
       <c r="F52" s="17" t="inlineStr">
@@ -15446,51 +15326,47 @@
       </c>
       <c r="J52" s="17" t="inlineStr">
         <is>
+          <t>OEM СберАвто финал (15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="17" t="inlineStr">
+        <is>
+          <t>Форвард Авто Лада Ижевск</t>
+        </is>
+      </c>
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>ONLINE ФОРВАРД Авто Ижевск (ООО "ФОРВАРД-АВТО")</t>
+        </is>
+      </c>
+      <c r="D53" s="16" t="inlineStr"/>
+      <c r="E53" s="17" t="inlineStr">
+        <is>
+          <t>РФ</t>
+        </is>
+      </c>
+      <c r="F53" s="17" t="inlineStr">
+        <is>
+          <t>LADA</t>
+        </is>
+      </c>
+      <c r="G53" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J53" s="17" t="inlineStr">
+        <is>
           <t>Сделки Сентябрь 2026 (Битрикс)</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="4" t="n">
-        <v>49</v>
-      </c>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">	ФДЦ АВТОЦЕНТР НА ЗАВОДСКОМ Самара</t>
-        </is>
-      </c>
-      <c r="C53" s="7" t="inlineStr">
-        <is>
-          <t>АВТОЦЕНТР НА ЗАВОДСКОМ</t>
-        </is>
-      </c>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>6318143548</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="inlineStr">
-        <is>
-          <t>Самара</t>
-        </is>
-      </c>
-      <c r="F53" s="7" t="inlineStr">
-        <is>
-          <t>LADA</t>
-        </is>
-      </c>
-      <c r="G53" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H53" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I53" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J53" s="7" t="inlineStr">
-        <is>
-          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -15500,23 +15376,27 @@
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>CHERY/TENET Нижегородец</t>
+          <t xml:space="preserve">	ФДЦ АВТОЦЕНТР НА ЗАВОДСКОМ Самара</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Нижегородец, СберАвто</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr"/>
+          <t>АВТОЦЕНТР НА ЗАВОДСКОМ</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>6318143548</t>
+        </is>
+      </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Самара</t>
         </is>
       </c>
       <c r="F54" s="11" t="inlineStr">
         <is>
-          <t>CHERY &amp; TENET</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G54" s="10" t="n">
@@ -15530,7 +15410,7 @@
       </c>
       <c r="J54" s="11" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -15540,27 +15420,23 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>JETOUR Мотом</t>
+          <t>CHERY/TENET Нижегородец</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>JETOUR Мотом</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>7327045193</t>
-        </is>
-      </c>
+          <t>СберАвто, Нижегородец</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr"/>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>Ульяновск</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>CHERY &amp; TENET</t>
         </is>
       </c>
       <c r="G55" s="6" t="n">
@@ -15574,7 +15450,7 @@
       </c>
       <c r="J55" s="7" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -15584,22 +15460,22 @@
       </c>
       <c r="B56" s="11" t="inlineStr">
         <is>
-          <t>Jetour Планета Авто</t>
+          <t>JETOUR Мотом</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Jetour Планета Авто</t>
+          <t>JETOUR Мотом</t>
         </is>
       </c>
       <c r="D56" s="8" t="inlineStr">
         <is>
-          <t>7452048272</t>
+          <t>7327045193</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>Челябинск</t>
+          <t>Ульяновск</t>
         </is>
       </c>
       <c r="F56" s="11" t="inlineStr">
@@ -15628,12 +15504,12 @@
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Jetour Планета Авто Миасс</t>
+          <t>Jetour Планета Авто</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Jetour Планета Авто Миасс</t>
+          <t>Jetour Планета Авто</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -15643,7 +15519,7 @@
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>Челябинск область</t>
+          <t>Челябинск</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
@@ -15672,27 +15548,27 @@
       </c>
       <c r="B58" s="11" t="inlineStr">
         <is>
-          <t>Авто-Моторс</t>
+          <t>Jetour Планета Авто Миасс</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Авто-Моторс</t>
+          <t>Jetour Планета Авто Миасс</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr">
         <is>
-          <t>8602240702</t>
+          <t>7452048272</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>Сургут</t>
+          <t>Челябинск область</t>
         </is>
       </c>
       <c r="F58" s="11" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G58" s="10" t="n">
@@ -15716,27 +15592,27 @@
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>АвтоМаркет Jetour</t>
+          <t>Авто-Моторс</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>АвтоМаркет</t>
+          <t>Авто-Моторс</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>1841096486</t>
+          <t>8602240702</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>Ижевск</t>
+          <t>Сургут</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G59" s="6" t="n">
@@ -15760,27 +15636,27 @@
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>АГАТ-АВТО</t>
+          <t>АвтоМаркет Jetour</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>АГАТ-АВТО</t>
+          <t>АвтоМаркет</t>
         </is>
       </c>
       <c r="D60" s="8" t="inlineStr">
         <is>
-          <t>3804048079</t>
+          <t>1841096486</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
         <is>
-          <t>Иркутск</t>
+          <t>Ижевск</t>
         </is>
       </c>
       <c r="F60" s="11" t="inlineStr">
         <is>
-          <t>OMODA</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G60" s="10" t="n">
@@ -15804,27 +15680,27 @@
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>АМК-Екатеринбург</t>
+          <t>АГАТ-АВТО</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>АМК-Екатеринбург</t>
+          <t>АГАТ-АВТО</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>6672171350</t>
+          <t>3804048079</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>Екатеринбург</t>
+          <t>Иркутск</t>
         </is>
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>OMODA</t>
         </is>
       </c>
       <c r="G61" s="6" t="n">
@@ -15848,12 +15724,12 @@
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>АМК-Екатеринбург Серов</t>
+          <t>АМК-Екатеринбург</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>АМК-Екатеринбург Серов</t>
+          <t>АМК-Екатеринбург</t>
         </is>
       </c>
       <c r="D62" s="8" t="inlineStr">
@@ -15892,27 +15768,27 @@
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Армада Авто</t>
+          <t>АМК-Екатеринбург Серов</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>Армада Авто</t>
+          <t>АМК-Екатеринбург Серов</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>7327075832</t>
+          <t>6672171350</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>Ульяновск</t>
+          <t>Екатеринбург</t>
         </is>
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G63" s="6" t="n">
@@ -15936,27 +15812,27 @@
       </c>
       <c r="B64" s="11" t="inlineStr">
         <is>
-          <t>БЦР</t>
+          <t>Армада Авто</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>БЦР</t>
+          <t>Армада Авто</t>
         </is>
       </c>
       <c r="D64" s="8" t="inlineStr">
         <is>
-          <t>5610251967</t>
+          <t>7327075832</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
-          <t>Нижний Новгород</t>
+          <t>Ульяновск</t>
         </is>
       </c>
       <c r="F64" s="11" t="inlineStr">
         <is>
-          <t>CHANGAN</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G64" s="10" t="n">
@@ -15980,27 +15856,27 @@
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>ГК Автобан Джетур</t>
+          <t>БЦР</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>ГК Автобан Джетур</t>
+          <t>БЦР</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>6679163711</t>
+          <t>5610251967</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>Екатеринбург</t>
+          <t>Нижний Новгород</t>
         </is>
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>CHANGAN</t>
         </is>
       </c>
       <c r="G65" s="6" t="n">
@@ -16024,17 +15900,17 @@
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>ГК Глазурит</t>
+          <t>ГК Автобан Джетур</t>
         </is>
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>ГК Глазурит</t>
+          <t>ГК Автобан Джетур</t>
         </is>
       </c>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>6626011680</t>
+          <t>6679163711</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
@@ -16068,22 +15944,22 @@
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>ГК Дактор Уфа</t>
+          <t>ГК Глазурит</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>ГК Дактор Уфа</t>
+          <t>ГК Глазурит</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>0276971419</t>
+          <t>6626011680</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>Уфа</t>
+          <t>Екатеринбург</t>
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr">
@@ -16112,27 +15988,27 @@
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
-          <t>ГК Колесо</t>
+          <t>ГК Дактор Уфа</t>
         </is>
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>ГК Колесо</t>
+          <t>ГК Дактор Уфа</t>
         </is>
       </c>
       <c r="D68" s="8" t="inlineStr">
         <is>
-          <t>3025026743</t>
+          <t>0276971419</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>Астрахань</t>
+          <t>Уфа</t>
         </is>
       </c>
       <c r="F68" s="11" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G68" s="10" t="n">
@@ -16156,27 +16032,27 @@
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>ГК Лаки Моторс Джетур</t>
+          <t>ГК Колесо</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>ГК Лаки Моторс Джетур</t>
+          <t>ГК Колесо</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>6664044905</t>
+          <t>3025026743</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>Екатеринбург</t>
+          <t>Астрахань</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G69" s="6" t="n">
@@ -16200,17 +16076,17 @@
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>Глазурит Лада</t>
+          <t>ГК Лаки Моторс Джетур</t>
         </is>
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>Глазурит Лада</t>
+          <t>ГК Лаки Моторс Джетур</t>
         </is>
       </c>
       <c r="D70" s="8" t="inlineStr">
         <is>
-          <t>6686064831</t>
+          <t>6664044905</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
@@ -16220,7 +16096,7 @@
       </c>
       <c r="F70" s="11" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G70" s="10" t="n">
@@ -16244,27 +16120,27 @@
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>Дав Авто</t>
+          <t>Глазурит Лада</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>Дав Авто</t>
+          <t>Глазурит Лада</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>5904329207</t>
+          <t>6686064831</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>Пермь</t>
+          <t>Екатеринбург</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>GEELY,BELGEE,KNEWSTAR</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G71" s="6" t="n">
@@ -16298,7 +16174,7 @@
       </c>
       <c r="D72" s="8" t="inlineStr">
         <is>
-          <t>5905016567</t>
+          <t>5904329207</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
@@ -16308,7 +16184,7 @@
       </c>
       <c r="F72" s="11" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>GEELY,BELGEE,KNEWSTAR</t>
         </is>
       </c>
       <c r="G72" s="10" t="n">
@@ -16332,27 +16208,27 @@
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>Интерпартнер</t>
+          <t>Дав Авто</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>Чери Центр Интерпартнер</t>
+          <t>Дав Авто</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>1835035118</t>
+          <t>5905016567</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>Ижевск</t>
+          <t>Пермь</t>
         </is>
       </c>
       <c r="F73" s="7" t="inlineStr">
         <is>
-          <t>CHERY</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G73" s="6" t="n">
@@ -16376,27 +16252,27 @@
       </c>
       <c r="B74" s="11" t="inlineStr">
         <is>
-          <t>Колесо Астрахань</t>
+          <t>Интерпартнер</t>
         </is>
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>Колесо</t>
+          <t>Чери Центр Интерпартнер</t>
         </is>
       </c>
       <c r="D74" s="8" t="inlineStr">
         <is>
-          <t>3025026743</t>
+          <t>1835035118</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
         <is>
-          <t>Астрахань</t>
+          <t>Ижевск</t>
         </is>
       </c>
       <c r="F74" s="11" t="inlineStr">
         <is>
-          <t>SOLARIS</t>
+          <t>CHERY</t>
         </is>
       </c>
       <c r="G74" s="10" t="n">
@@ -16420,27 +16296,27 @@
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>Комос-Авто</t>
+          <t>Колесо Астрахань</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>Комос-Авто</t>
+          <t>Колесо</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>1831088285</t>
+          <t>3025026743</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>Ижевск</t>
+          <t>Астрахань</t>
         </is>
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>GEELY,KNEWSTAR</t>
+          <t>SOLARIS</t>
         </is>
       </c>
       <c r="G75" s="6" t="n">
@@ -16464,27 +16340,27 @@
       </c>
       <c r="B76" s="11" t="inlineStr">
         <is>
-          <t>Курган Лдетур Оками</t>
+          <t>Комос-Авто</t>
         </is>
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>Курган Лдетур Оками</t>
+          <t>Комос-Авто</t>
         </is>
       </c>
       <c r="D76" s="8" t="inlineStr">
         <is>
-          <t>6606034288</t>
+          <t>1831088285</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
         <is>
-          <t>Курган</t>
+          <t>Ижевск</t>
         </is>
       </c>
       <c r="F76" s="11" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>GEELY,KNEWSTAR</t>
         </is>
       </c>
       <c r="G76" s="10" t="n">
@@ -16508,27 +16384,27 @@
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>Мерит</t>
+          <t>Курган Лдетур Оками</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>Мерит</t>
+          <t>Курган Лдетур Оками</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>6330079024</t>
+          <t>6606034288</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>Самарская обл., г. Новокуйбышевск</t>
+          <t>Курган</t>
         </is>
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G77" s="6" t="n">
@@ -16552,22 +16428,22 @@
       </c>
       <c r="B78" s="11" t="inlineStr">
         <is>
-          <t>Олимп Уфа</t>
+          <t>Мерит</t>
         </is>
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>Олимп Уфа</t>
+          <t>Мерит</t>
         </is>
       </c>
       <c r="D78" s="8" t="inlineStr">
         <is>
-          <t>2311093925</t>
+          <t>6330079024</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
         <is>
-          <t>Уфа</t>
+          <t>Самарская обл., г. Новокуйбышевск</t>
         </is>
       </c>
       <c r="F78" s="11" t="inlineStr">
@@ -16596,18 +16472,22 @@
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>пилот ФДЦ Автосеть РФ АМК Самара Тольятти ЕКБ</t>
+          <t>Олимп Уфа</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>ONLINE  пилот ФДЦ Автосеть РФ АМК Самара Тольятти ЕКБ</t>
-        </is>
-      </c>
-      <c r="D79" s="4" t="inlineStr"/>
+          <t>Олимп Уфа</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>2311093925</t>
+        </is>
+      </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Уфа</t>
         </is>
       </c>
       <c r="F79" s="7" t="inlineStr">
@@ -16626,7 +16506,7 @@
       </c>
       <c r="J79" s="7" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -16636,27 +16516,23 @@
       </c>
       <c r="B80" s="11" t="inlineStr">
         <is>
-          <t>Планета Авто</t>
+          <t>пилот ФДЦ Автосеть РФ АМК Самара Тольятти ЕКБ</t>
         </is>
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>Планета Авто</t>
-        </is>
-      </c>
-      <c r="D80" s="8" t="inlineStr">
-        <is>
-          <t>7452048272</t>
-        </is>
-      </c>
+          <t>ONLINE  пилот ФДЦ Автосеть РФ АМК Самара Тольятти ЕКБ</t>
+        </is>
+      </c>
+      <c r="D80" s="8" t="inlineStr"/>
       <c r="E80" s="11" t="inlineStr">
         <is>
-          <t>Челябинск</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F80" s="11" t="inlineStr">
         <is>
-          <t>OMODA</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G80" s="10" t="n">
@@ -16670,7 +16546,7 @@
       </c>
       <c r="J80" s="11" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -16680,27 +16556,27 @@
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>Русская Ладья</t>
+          <t>Планета Авто</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>Русская Ладья</t>
+          <t>Планета Авто</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>1831158253</t>
+          <t>7452048272</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>Ижевск</t>
+          <t>Челябинск</t>
         </is>
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>OMODA</t>
         </is>
       </c>
       <c r="G81" s="6" t="n">
@@ -16724,22 +16600,22 @@
       </c>
       <c r="B82" s="11" t="inlineStr">
         <is>
-          <t>Самара - Лада</t>
+          <t>Русская Ладья</t>
         </is>
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>Самара - Лада</t>
+          <t>Русская Ладья</t>
         </is>
       </c>
       <c r="D82" s="8" t="inlineStr">
         <is>
-          <t>6312012764</t>
+          <t>1831158253</t>
         </is>
       </c>
       <c r="E82" s="11" t="inlineStr">
         <is>
-          <t>Самара</t>
+          <t>Ижевск</t>
         </is>
       </c>
       <c r="F82" s="11" t="inlineStr">
@@ -16768,27 +16644,27 @@
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>Сатурн Р</t>
+          <t>Самара - Лада</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>Сатурн Р</t>
+          <t>Самара - Лада</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>5902809279</t>
+          <t>6312012764</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>Пермь</t>
+          <t>Самара</t>
         </is>
       </c>
       <c r="F83" s="7" t="inlineStr">
         <is>
-          <t>OMODA</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G83" s="6" t="n">
@@ -16812,27 +16688,27 @@
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>Сатурн-2</t>
+          <t>Сатурн Р</t>
         </is>
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>Tenet Сатурн-2</t>
+          <t>Сатурн Р</t>
         </is>
       </c>
       <c r="D84" s="8" t="inlineStr">
         <is>
-          <t>7449019666</t>
+          <t>5902809279</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
         <is>
-          <t>Челябинск</t>
+          <t>Пермь</t>
         </is>
       </c>
       <c r="F84" s="11" t="inlineStr">
         <is>
-          <t>CHERY</t>
+          <t>OMODA</t>
         </is>
       </c>
       <c r="G84" s="10" t="n">
@@ -16856,27 +16732,27 @@
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>ТД Армада Авто Джетур</t>
+          <t>Сатурн-2</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>ТД Армада Авто Джетур</t>
+          <t>Tenet Сатурн-2</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>7327075832</t>
+          <t>7449019666</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>УФА</t>
+          <t>Челябинск</t>
         </is>
       </c>
       <c r="F85" s="7" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>CHERY</t>
         </is>
       </c>
       <c r="G85" s="6" t="n">
@@ -16900,27 +16776,27 @@
       </c>
       <c r="B86" s="11" t="inlineStr">
         <is>
-          <t>Ункиум</t>
+          <t>ТД Армада Авто Джетур</t>
         </is>
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>Ункиум</t>
+          <t>ТД Армада Авто Джетур</t>
         </is>
       </c>
       <c r="D86" s="8" t="inlineStr">
         <is>
-          <t>6678064041</t>
+          <t>7327075832</t>
         </is>
       </c>
       <c r="E86" s="11" t="inlineStr">
         <is>
-          <t>Екатеринбург</t>
+          <t>УФА</t>
         </is>
       </c>
       <c r="F86" s="11" t="inlineStr">
         <is>
-          <t>CHERY</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G86" s="10" t="n">
@@ -16944,27 +16820,27 @@
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>Урал Лада Красный Яр</t>
+          <t>Ункиум</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>Урал Лада Красный Яр</t>
+          <t>Ункиум</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>6376003892</t>
+          <t>6678064041</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>Самара</t>
+          <t>Екатеринбург</t>
         </is>
       </c>
       <c r="F87" s="7" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>CHERY</t>
         </is>
       </c>
       <c r="G87" s="6" t="n">
@@ -16988,12 +16864,12 @@
       </c>
       <c r="B88" s="11" t="inlineStr">
         <is>
-          <t>Урал Лада Самара</t>
+          <t>Урал Лада Красный Яр</t>
         </is>
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>Урал Лада Самара</t>
+          <t>Урал Лада Красный Яр</t>
         </is>
       </c>
       <c r="D88" s="8" t="inlineStr">
@@ -17032,27 +16908,27 @@
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>Уфа Haval Автопремьер М</t>
+          <t>Урал Лада Самара</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>Уфа Haval Автопремьер М</t>
+          <t>Урал Лада Самара</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>0273059765</t>
+          <t>6376003892</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>Уфа</t>
+          <t>Самара</t>
         </is>
       </c>
       <c r="F89" s="7" t="inlineStr">
         <is>
-          <t>HAVAL</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G89" s="6" t="n">
@@ -17076,27 +16952,27 @@
       </c>
       <c r="B90" s="11" t="inlineStr">
         <is>
-          <t>ФДЦ ОСА-Холдинг г. Бузулук Оренбургская обл.</t>
+          <t>Уфа Haval Автопремьер М</t>
         </is>
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>ОСА-Холдинг</t>
+          <t>Уфа Haval Автопремьер М</t>
         </is>
       </c>
       <c r="D90" s="8" t="inlineStr">
         <is>
-          <t>5603013320</t>
+          <t>0273059765</t>
         </is>
       </c>
       <c r="E90" s="11" t="inlineStr">
         <is>
-          <t>Оренбургская обл., г. Бузулук</t>
+          <t>Уфа</t>
         </is>
       </c>
       <c r="F90" s="11" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>HAVAL</t>
         </is>
       </c>
       <c r="G90" s="10" t="n">
@@ -17120,18 +16996,22 @@
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>Форвард  Ижевск/Сызрань</t>
+          <t>ФДЦ ОСА-Холдинг г. Бузулук Оренбургская обл.</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>ONLINE Форвард  Ижевск/Сызрань</t>
-        </is>
-      </c>
-      <c r="D91" s="4" t="inlineStr"/>
+          <t>ОСА-Холдинг</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>5603013320</t>
+        </is>
+      </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Оренбургская обл., г. Бузулук</t>
         </is>
       </c>
       <c r="F91" s="7" t="inlineStr">
@@ -17150,7 +17030,7 @@
       </c>
       <c r="J91" s="7" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -17160,22 +17040,18 @@
       </c>
       <c r="B92" s="11" t="inlineStr">
         <is>
-          <t>Центральное СТО 50 лет Октября</t>
+          <t>Форвард  Ижевск/Сызрань</t>
         </is>
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>Центральное СТО 50 лет Октября</t>
-        </is>
-      </c>
-      <c r="D92" s="8" t="inlineStr">
-        <is>
-          <t>6320011130</t>
-        </is>
-      </c>
+          <t>ONLINE Форвард  Ижевск/Сызрань</t>
+        </is>
+      </c>
+      <c r="D92" s="8" t="inlineStr"/>
       <c r="E92" s="11" t="inlineStr">
         <is>
-          <t>Тольятти</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F92" s="11" t="inlineStr">
@@ -17194,7 +17070,7 @@
       </c>
       <c r="J92" s="11" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -17204,12 +17080,12 @@
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>Центральное СТО на Громова</t>
+          <t>Центральное СТО 50 лет Октября</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>Центральное СТО на Громова</t>
+          <t>Центральное СТО 50 лет Октября</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -17248,12 +17124,12 @@
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>Центральное СТО на Южном ш.</t>
+          <t>Центральное СТО на Громова</t>
         </is>
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>Центральное СТО на Южном ш.</t>
+          <t>Центральное СТО на Громова</t>
         </is>
       </c>
       <c r="D94" s="8" t="inlineStr">
@@ -17292,27 +17168,27 @@
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>Чанган Центр АВТОФОРУМ ВОСТОК</t>
+          <t>Центральное СТО на Южном ш.</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>Чанган Центр АВТОФОРУМ ВОСТОК</t>
+          <t>Центральное СТО на Южном ш.</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>6453163950</t>
+          <t>6320011130</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>Саратов</t>
+          <t>Тольятти</t>
         </is>
       </c>
       <c r="F95" s="7" t="inlineStr">
         <is>
-          <t>CHANGAN</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G95" s="6" t="n">
@@ -17336,27 +17212,27 @@
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>Чери Арконт</t>
+          <t>Чанган Центр АВТОФОРУМ ВОСТОК</t>
         </is>
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>Чери Арконт</t>
+          <t>Чанган Центр АВТОФОРУМ ВОСТОК</t>
         </is>
       </c>
       <c r="D96" s="8" t="inlineStr">
         <is>
-          <t>3443089821</t>
+          <t>6453163950</t>
         </is>
       </c>
       <c r="E96" s="11" t="inlineStr">
         <is>
-          <t>Волгоград</t>
+          <t>Саратов</t>
         </is>
       </c>
       <c r="F96" s="11" t="inlineStr">
         <is>
-          <t>CHERY</t>
+          <t>CHANGAN</t>
         </is>
       </c>
       <c r="G96" s="10" t="n">
@@ -17380,22 +17256,22 @@
       </c>
       <c r="B97" s="7" t="inlineStr">
         <is>
-          <t>ЧЕРИ ЦЕНТР ВИП АВТО САМАРА ОНЛАЙН</t>
+          <t>Чери Арконт</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>ЧЕРИ ЦЕНТР ВИП АВТО САМАРА ОНЛАЙН</t>
+          <t>Чери Арконт</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>6312214182</t>
+          <t>3443089821</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>Самара</t>
+          <t>Волгоград</t>
         </is>
       </c>
       <c r="F97" s="7" t="inlineStr">
@@ -17424,22 +17300,22 @@
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>ЧЕРИ ЦЕНТР ЭКСКУРС ПЕРМЬ ОНЛАЙН</t>
+          <t>ЧЕРИ ЦЕНТР ВИП АВТО САМАРА ОНЛАЙН</t>
         </is>
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>ЧЕРИ ЦЕНТР ЭКСКУРС ПЕРМЬ ОНЛАЙН</t>
+          <t>ЧЕРИ ЦЕНТР ВИП АВТО САМАРА ОНЛАЙН</t>
         </is>
       </c>
       <c r="D98" s="8" t="inlineStr">
         <is>
-          <t>5903101739</t>
+          <t>6312214182</t>
         </is>
       </c>
       <c r="E98" s="11" t="inlineStr">
         <is>
-          <t>Пермь</t>
+          <t>Самара</t>
         </is>
       </c>
       <c r="F98" s="11" t="inlineStr">
@@ -17468,75 +17344,119 @@
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
+          <t>ЧЕРИ ЦЕНТР ЭКСКУРС ПЕРМЬ ОНЛАЙН</t>
+        </is>
+      </c>
+      <c r="C99" s="7" t="inlineStr">
+        <is>
+          <t>ЧЕРИ ЦЕНТР ЭКСКУРС ПЕРМЬ ОНЛАЙН</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>5903101739</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="inlineStr">
+        <is>
+          <t>Пермь</t>
+        </is>
+      </c>
+      <c r="F99" s="7" t="inlineStr">
+        <is>
+          <t>CHERY</t>
+        </is>
+      </c>
+      <c r="G99" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I99" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J99" s="7" t="inlineStr">
+        <is>
+          <t>OEM СберАвто финал (15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="20" customHeight="1">
+      <c r="A100" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="B100" s="11" t="inlineStr">
+        <is>
           <t>Эксперт Альфа Джетур</t>
         </is>
       </c>
-      <c r="C99" s="7" t="inlineStr">
+      <c r="C100" s="11" t="inlineStr">
         <is>
           <t>Эксперт Альфа Джетур</t>
         </is>
       </c>
-      <c r="D99" s="4" t="inlineStr">
+      <c r="D100" s="8" t="inlineStr">
         <is>
           <t>9709054813</t>
         </is>
       </c>
-      <c r="E99" s="7" t="inlineStr">
+      <c r="E100" s="11" t="inlineStr">
         <is>
           <t>Самара</t>
         </is>
       </c>
-      <c r="F99" s="7" t="inlineStr">
+      <c r="F100" s="11" t="inlineStr">
         <is>
           <t>JETOUR</t>
         </is>
       </c>
-      <c r="G99" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H99" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I99" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J99" s="7" t="inlineStr">
-        <is>
-          <t>OEM СберАвто финал (15)</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="24" customHeight="1">
-      <c r="A100" s="12" t="inlineStr"/>
-      <c r="B100" s="13" t="inlineStr">
+      <c r="G100" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I100" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J100" s="11" t="inlineStr">
+        <is>
+          <t>OEM СберАвто финал (15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="24" customHeight="1">
+      <c r="A101" s="12" t="inlineStr"/>
+      <c r="B101" s="13" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="C100" s="13" t="inlineStr">
-        <is>
-          <t>95 объектов</t>
-        </is>
-      </c>
-      <c r="D100" s="12" t="n"/>
-      <c r="E100" s="12" t="n"/>
-      <c r="F100" s="12" t="n"/>
-      <c r="G100" s="14">
-        <f>SUM(G5:G99)</f>
+      <c r="C101" s="13" t="inlineStr">
+        <is>
+          <t>96 объектов</t>
+        </is>
+      </c>
+      <c r="D101" s="12" t="n"/>
+      <c r="E101" s="12" t="n"/>
+      <c r="F101" s="12" t="n"/>
+      <c r="G101" s="14">
+        <f>SUM(G5:G100)</f>
         <v/>
       </c>
-      <c r="H100" s="14">
-        <f>SUM(H5:H99)</f>
+      <c r="H101" s="14">
+        <f>SUM(H5:H100)</f>
         <v/>
       </c>
-      <c r="I100" s="14">
-        <f>SUM(I5:I99)</f>
+      <c r="I101" s="14">
+        <f>SUM(I5:I100)</f>
         <v/>
       </c>
-      <c r="J100" s="12" t="n"/>
+      <c r="J101" s="12" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J99"/>
+  <autoFilter ref="A4:J100"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17552,7 +17472,7 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="41" customWidth="1" min="2" max="2"/>
-    <col width="69" customWidth="1" min="3" max="3"/>
+    <col width="91" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -18560,7 +18480,7 @@
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>ООО "ДИНАМИКА АРХАНГЕЛЬСК" ONLINE, ООО "ДИНАМИКА ЧЕРЕПОВЕЦ" ONLINE</t>
+          <t>ООО "ДИНАМИКА ЧЕРЕПОВЕЦ" ONLINE, СберАвто</t>
         </is>
       </c>
       <c r="D26" s="16" t="inlineStr"/>
@@ -18743,7 +18663,7 @@
       </c>
       <c r="F30" s="17" t="inlineStr">
         <is>
-          <t>SOUEAST, LADA</t>
+          <t>LADA, SOUEAST</t>
         </is>
       </c>
       <c r="G30" s="18" t="n">
@@ -19556,7 +19476,7 @@
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>ONLINE Пилот ФДЦ Прагматика СпБ В-НГРД ПСКВ, Атик</t>
+          <t>ONLINE Прагматика (ООО Прагматика Мурманск), ONLINE Пилот ФДЦ Прагматика СпБ В-НГРД ПСКВ</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr"/>
@@ -19567,7 +19487,7 @@
       </c>
       <c r="F49" s="17" t="inlineStr">
         <is>
-          <t>OMODA &amp; JAECOO, LADA</t>
+          <t>LADA, OMODA &amp; JAECOO</t>
         </is>
       </c>
       <c r="G49" s="18" t="n">
@@ -20146,44 +20066,44 @@
       </c>
     </row>
     <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="16" t="n">
+      <c r="A63" s="4" t="n">
         <v>59</v>
       </c>
-      <c r="B63" s="17" t="inlineStr">
-        <is>
-          <t>Форвард</t>
-        </is>
-      </c>
-      <c r="C63" s="17" t="inlineStr">
-        <is>
-          <t>Чери Центр Форвард-Авто</t>
-        </is>
-      </c>
-      <c r="D63" s="16" t="inlineStr">
-        <is>
-          <t>5906145075</t>
-        </is>
-      </c>
-      <c r="E63" s="17" t="inlineStr">
-        <is>
-          <t>Тюмень</t>
-        </is>
-      </c>
-      <c r="F63" s="17" t="inlineStr">
-        <is>
-          <t>CHERY</t>
-        </is>
-      </c>
-      <c r="G63" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="H63" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I63" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="J63" s="17" t="inlineStr">
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>ONLIN Авто Премиум Тверь</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Авто Премиум</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>7802455157</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>JETOUR</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" s="7" t="inlineStr">
         <is>
           <t>OEM СберАвто финал (15)</t>
         </is>
@@ -20215,7 +20135,7 @@
       </c>
       <c r="F64" s="11" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>SOUEAST</t>
         </is>
       </c>
       <c r="G64" s="10" t="n">
@@ -20239,17 +20159,17 @@
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>ONLIN Авто Премиум Тверь</t>
+          <t>Tenet Элан-Моторс</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>Авто Премиум</t>
+          <t>Tenet Элан-Моторс</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>7802455157</t>
+          <t>7806289863</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
@@ -20259,7 +20179,7 @@
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>SOUEAST</t>
+          <t>CHERY</t>
         </is>
       </c>
       <c r="G65" s="6" t="n">
@@ -20283,27 +20203,27 @@
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>Tenet Элан-Моторс</t>
+          <t>АБМ</t>
         </is>
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>Tenet Элан-Моторс</t>
+          <t>АБМ</t>
         </is>
       </c>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>7806289863</t>
+          <t>5190003694</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
         <is>
-          <t>Санкт-Петербург</t>
+          <t>Мурманск</t>
         </is>
       </c>
       <c r="F66" s="11" t="inlineStr">
         <is>
-          <t>CHERY</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G66" s="10" t="n">
@@ -20347,7 +20267,7 @@
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>SOUEAST</t>
         </is>
       </c>
       <c r="G67" s="6" t="n">
@@ -20371,27 +20291,23 @@
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
-          <t>АБМ</t>
+          <t>Автомаг</t>
         </is>
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>АБМ</t>
-        </is>
-      </c>
-      <c r="D68" s="8" t="inlineStr">
-        <is>
-          <t>5190003694</t>
-        </is>
-      </c>
+          <t>Автомаг</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr"/>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>Мурманск</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F68" s="11" t="inlineStr">
         <is>
-          <t>SOUEAST</t>
+          <t>Geely, HAVAL</t>
         </is>
       </c>
       <c r="G68" s="10" t="n">
@@ -20405,7 +20321,7 @@
       </c>
       <c r="J68" s="11" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -20415,23 +20331,23 @@
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>Автомаг</t>
+          <t>Автомобильный Центр Псков</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Автомаг</t>
+          <t>Автомобильный Центр Псков</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr"/>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Псков</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>HAVAL, Geely</t>
+          <t>CHERY</t>
         </is>
       </c>
       <c r="G69" s="6" t="n">
@@ -20445,7 +20361,7 @@
       </c>
       <c r="J69" s="7" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -20455,18 +20371,22 @@
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>Автомобильный Центр Псков</t>
+          <t>Автопортрет</t>
         </is>
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>Автомобильный Центр Псков</t>
-        </is>
-      </c>
-      <c r="D70" s="8" t="inlineStr"/>
+          <t>Автопортрет</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>7810337380</t>
+        </is>
+      </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>Псков</t>
+          <t>Санкт-Петербург</t>
         </is>
       </c>
       <c r="F70" s="11" t="inlineStr">
@@ -20505,7 +20425,7 @@
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>7810337380</t>
+          <t>7816740073</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
@@ -20515,7 +20435,7 @@
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>CHERY</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G71" s="6" t="n">
@@ -20539,27 +20459,27 @@
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>Автопортрет</t>
+          <t>Автопортрет Про</t>
         </is>
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>Автопортрет</t>
+          <t>Автопортрет Про</t>
         </is>
       </c>
       <c r="D72" s="8" t="inlineStr">
         <is>
-          <t>7816740073</t>
+          <t>7810337380</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>Санкт-Петербург</t>
+          <t>Санк-Петербург</t>
         </is>
       </c>
       <c r="F72" s="11" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>HAVAL</t>
         </is>
       </c>
       <c r="G72" s="10" t="n">
@@ -20583,12 +20503,12 @@
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>Автопортрет Про</t>
+          <t>Автопортрет Сити</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>Автопортрет Про</t>
+          <t>Автопортрет Сити</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -20637,7 +20557,7 @@
       </c>
       <c r="D74" s="8" t="inlineStr">
         <is>
-          <t>7810337380</t>
+          <t>7814693364</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
@@ -20671,27 +20591,27 @@
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>Автопортрет Сити</t>
+          <t>Авторитэйл Выборгское</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>Автопортрет Сити</t>
+          <t>Авторитэйл Выборгское</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>7814693364</t>
+          <t>7801214832</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>Санк-Петербург</t>
+          <t>Санкт-Петербург</t>
         </is>
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>HAVAL</t>
+          <t>CHANGAN</t>
         </is>
       </c>
       <c r="G75" s="6" t="n">
@@ -20715,12 +20635,12 @@
       </c>
       <c r="B76" s="11" t="inlineStr">
         <is>
-          <t>Авторитэйл Выборгское</t>
+          <t>Авторитэйл Таллинское</t>
         </is>
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>Авторитэйл Выборгское</t>
+          <t>Авторитэйл Таллинское</t>
         </is>
       </c>
       <c r="D76" s="8" t="inlineStr">
@@ -20779,7 +20699,7 @@
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>CHANGAN</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G77" s="6" t="n">
@@ -20803,27 +20723,27 @@
       </c>
       <c r="B78" s="11" t="inlineStr">
         <is>
-          <t>Авторитэйл Таллинское</t>
+          <t>Автосалон № 1</t>
         </is>
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>Авторитэйл Таллинское</t>
+          <t>Автосалон № 1</t>
         </is>
       </c>
       <c r="D78" s="8" t="inlineStr">
         <is>
-          <t>7801214832</t>
+          <t>6000005056</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
         <is>
-          <t>Санкт-Петербург</t>
+          <t>Псков</t>
         </is>
       </c>
       <c r="F78" s="11" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>CHERY</t>
         </is>
       </c>
       <c r="G78" s="10" t="n">
@@ -20847,22 +20767,22 @@
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>Автосалон № 1</t>
+          <t>Автостиль Чери Новгород</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>Автосалон № 1</t>
+          <t>Автостиль Чери Новгород</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>6000005056</t>
+          <t>7805752165</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>Псков</t>
+          <t>Великий Новгород</t>
         </is>
       </c>
       <c r="F79" s="7" t="inlineStr">
@@ -20891,12 +20811,12 @@
       </c>
       <c r="B80" s="11" t="inlineStr">
         <is>
-          <t>Автостиль Чери Новгород</t>
+          <t>Автостиль Чери СПБ</t>
         </is>
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>Автостиль Чери Новгород</t>
+          <t>Автостиль Чери СПБ</t>
         </is>
       </c>
       <c r="D80" s="8" t="inlineStr">
@@ -20906,7 +20826,7 @@
       </c>
       <c r="E80" s="11" t="inlineStr">
         <is>
-          <t>Великий Новгород</t>
+          <t>Санкт-Петербург</t>
         </is>
       </c>
       <c r="F80" s="11" t="inlineStr">
@@ -20935,27 +20855,27 @@
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>Автостиль Чери СПБ</t>
+          <t>Агат-Авто</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>Автостиль Чери СПБ</t>
+          <t>Агат-Авто</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>7805752165</t>
+          <t>3804048079</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>Санкт-Петербург</t>
+          <t>Братск</t>
         </is>
       </c>
       <c r="F81" s="7" t="inlineStr">
         <is>
-          <t>CHERY</t>
+          <t>CHANGAN</t>
         </is>
       </c>
       <c r="G81" s="6" t="n">
@@ -20979,27 +20899,27 @@
       </c>
       <c r="B82" s="11" t="inlineStr">
         <is>
-          <t>Агат-Авто</t>
+          <t>Ай-Би-Эм</t>
         </is>
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>Агат-Авто</t>
+          <t>ЧЕРИ ЦЕНТР Ай-Би-Эм Юг</t>
         </is>
       </c>
       <c r="D82" s="8" t="inlineStr">
         <is>
-          <t>3804048079</t>
+          <t>4207055973</t>
         </is>
       </c>
       <c r="E82" s="11" t="inlineStr">
         <is>
-          <t>Братск</t>
+          <t>Кемерово</t>
         </is>
       </c>
       <c r="F82" s="11" t="inlineStr">
         <is>
-          <t>CHANGAN</t>
+          <t>CHERY</t>
         </is>
       </c>
       <c r="G82" s="10" t="n">
@@ -21028,7 +20948,7 @@
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>ЧЕРИ ЦЕНТР Ай-Би-Эм Юг</t>
+          <t>Ай-Би-Эм</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -21043,7 +20963,7 @@
       </c>
       <c r="F83" s="7" t="inlineStr">
         <is>
-          <t>CHERY</t>
+          <t>GEELY,KNEWSTAR</t>
         </is>
       </c>
       <c r="G83" s="6" t="n">
@@ -21067,27 +20987,27 @@
       </c>
       <c r="B84" s="11" t="inlineStr">
         <is>
-          <t>Ай-Би-Эм</t>
+          <t>Аларм Моторс</t>
         </is>
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>Ай-Би-Эм</t>
+          <t>Аларм Моторс</t>
         </is>
       </c>
       <c r="D84" s="8" t="inlineStr">
         <is>
-          <t>4207055973</t>
+          <t>7802383738</t>
         </is>
       </c>
       <c r="E84" s="11" t="inlineStr">
         <is>
-          <t>Кемерово</t>
+          <t>Санкт-Петербург</t>
         </is>
       </c>
       <c r="F84" s="11" t="inlineStr">
         <is>
-          <t>GEELY,KNEWSTAR</t>
+          <t>CHERY</t>
         </is>
       </c>
       <c r="G84" s="10" t="n">
@@ -21165,7 +21085,7 @@
       </c>
       <c r="D86" s="8" t="inlineStr">
         <is>
-          <t>7802383738</t>
+          <t>7807166046</t>
         </is>
       </c>
       <c r="E86" s="11" t="inlineStr">
@@ -21175,7 +21095,7 @@
       </c>
       <c r="F86" s="11" t="inlineStr">
         <is>
-          <t>CHERY</t>
+          <t>SOLARIS</t>
         </is>
       </c>
       <c r="G86" s="10" t="n">
@@ -21199,17 +21119,17 @@
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>Аларм Моторс</t>
+          <t>Аларм-Моторс Лада</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>Аларм Моторс</t>
+          <t>Аларм-Моторс Лада</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>7807166046</t>
+          <t>7814626865</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
@@ -21219,7 +21139,7 @@
       </c>
       <c r="F87" s="7" t="inlineStr">
         <is>
-          <t>SOLARIS</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G87" s="6" t="n">
@@ -21243,17 +21163,17 @@
       </c>
       <c r="B88" s="11" t="inlineStr">
         <is>
-          <t>Аларм-Моторс Лада</t>
+          <t>Аларм-Моторс Сити Савушкина</t>
         </is>
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>Аларм-Моторс Лада</t>
+          <t>Аларм-Моторс Сити Савушкина</t>
         </is>
       </c>
       <c r="D88" s="8" t="inlineStr">
         <is>
-          <t>7814626865</t>
+          <t>7802383738</t>
         </is>
       </c>
       <c r="E88" s="11" t="inlineStr">
@@ -21263,7 +21183,7 @@
       </c>
       <c r="F88" s="11" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>HAVAL</t>
         </is>
       </c>
       <c r="G88" s="10" t="n">
@@ -21287,27 +21207,27 @@
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>Аларм-Моторс Сити Савушкина</t>
+          <t>Алгоритм-Сервис</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>Аларм-Моторс Сити Савушкина</t>
+          <t>Алгоритм-Сервис</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>7802383738</t>
+          <t>2901241358</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>Санкт-Петербург</t>
+          <t>Архангельск</t>
         </is>
       </c>
       <c r="F89" s="7" t="inlineStr">
         <is>
-          <t>HAVAL</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G89" s="6" t="n">
@@ -21331,27 +21251,27 @@
       </c>
       <c r="B90" s="11" t="inlineStr">
         <is>
-          <t>Алгоритм-Сервис</t>
+          <t>Базис Моторс</t>
         </is>
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>Алгоритм-Сервис</t>
+          <t>Базис Моторс</t>
         </is>
       </c>
       <c r="D90" s="8" t="inlineStr">
         <is>
-          <t>2901241358</t>
+          <t>7202212071</t>
         </is>
       </c>
       <c r="E90" s="11" t="inlineStr">
         <is>
-          <t>Архангельск</t>
+          <t>Тюмень</t>
         </is>
       </c>
       <c r="F90" s="11" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>GEELY,BELGEE,KNEWSTAR</t>
         </is>
       </c>
       <c r="G90" s="10" t="n">
@@ -21375,27 +21295,27 @@
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>Базис Моторс</t>
+          <t>Вагнер Авто (СПб)</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>Базис Моторс</t>
+          <t>Вагнер</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>7202212071</t>
+          <t>7801214832</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>Тюмень</t>
+          <t>Санкт-Петербург</t>
         </is>
       </c>
       <c r="F91" s="7" t="inlineStr">
         <is>
-          <t>GEELY,BELGEE,KNEWSTAR</t>
+          <t>DEEPAL</t>
         </is>
       </c>
       <c r="G91" s="6" t="n">
@@ -21419,17 +21339,17 @@
       </c>
       <c r="B92" s="11" t="inlineStr">
         <is>
-          <t>Вагнер Авто (СПб)</t>
+          <t>Город Русских Машин (ГРМ)</t>
         </is>
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>Вагнер</t>
+          <t>Город Русских Машин</t>
         </is>
       </c>
       <c r="D92" s="8" t="inlineStr">
         <is>
-          <t>7801214832</t>
+          <t>7805013573</t>
         </is>
       </c>
       <c r="E92" s="11" t="inlineStr">
@@ -21439,7 +21359,7 @@
       </c>
       <c r="F92" s="11" t="inlineStr">
         <is>
-          <t>DEEPAL</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G92" s="10" t="n">
@@ -21463,22 +21383,22 @@
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>Город Русских Машин (ГРМ)</t>
+          <t>Дюк и К</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>Город Русских Машин</t>
+          <t>Дюк и К</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>7805013573</t>
+          <t>4209032900</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>Санкт-Петербург</t>
+          <t>Кемерово</t>
         </is>
       </c>
       <c r="F93" s="7" t="inlineStr">
@@ -21507,27 +21427,27 @@
       </c>
       <c r="B94" s="11" t="inlineStr">
         <is>
-          <t>Дюк и К</t>
+          <t>Евросиб</t>
         </is>
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>Дюк и К</t>
+          <t>Евросиб</t>
         </is>
       </c>
       <c r="D94" s="8" t="inlineStr">
         <is>
-          <t>4209032900</t>
+          <t>4705065364</t>
         </is>
       </c>
       <c r="E94" s="11" t="inlineStr">
         <is>
-          <t>Кемерово</t>
+          <t>Санкт-Петербург</t>
         </is>
       </c>
       <c r="F94" s="11" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G94" s="10" t="n">
@@ -21551,27 +21471,23 @@
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>Евросиб</t>
+          <t>ЛАДА КУДРОВО</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>Евросиб</t>
-        </is>
-      </c>
-      <c r="D95" s="4" t="inlineStr">
-        <is>
-          <t>4705065364</t>
-        </is>
-      </c>
+          <t>Лада Кудрово</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr"/>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>Санкт-Петербург</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F95" s="7" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G95" s="6" t="n">
@@ -21585,7 +21501,7 @@
       </c>
       <c r="J95" s="7" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -21595,23 +21511,27 @@
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>ЛАДА КУДРОВО</t>
+          <t>Максимум Джили</t>
         </is>
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>Лада Кудрово</t>
-        </is>
-      </c>
-      <c r="D96" s="8" t="inlineStr"/>
+          <t>Максимум Джили</t>
+        </is>
+      </c>
+      <c r="D96" s="8" t="inlineStr">
+        <is>
+          <t>7804428906</t>
+        </is>
+      </c>
       <c r="E96" s="11" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Санк-Петербург</t>
         </is>
       </c>
       <c r="F96" s="11" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>GEELY</t>
         </is>
       </c>
       <c r="G96" s="10" t="n">
@@ -21625,7 +21545,7 @@
       </c>
       <c r="J96" s="11" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -21635,12 +21555,12 @@
       </c>
       <c r="B97" s="7" t="inlineStr">
         <is>
-          <t>Максимум Джили</t>
+          <t>Максимум Про</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>Максимум Джили</t>
+          <t>Максимум Про</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -21655,7 +21575,7 @@
       </c>
       <c r="F97" s="7" t="inlineStr">
         <is>
-          <t>GEELY</t>
+          <t>HAVAL</t>
         </is>
       </c>
       <c r="G97" s="6" t="n">
@@ -21679,12 +21599,12 @@
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>Максимум Про</t>
+          <t>Максимум Сити</t>
         </is>
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>Максимум Про</t>
+          <t>Максимум Сити</t>
         </is>
       </c>
       <c r="D98" s="8" t="inlineStr">
@@ -21723,27 +21643,27 @@
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
-          <t>Максимум Сити</t>
+          <t>Моторленд (Воронеж)</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>Максимум Сити</t>
+          <t>Моторленд</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>7804428906</t>
+          <t>3662259794</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>Санк-Петербург</t>
+          <t>Санкт-Петербург</t>
         </is>
       </c>
       <c r="F99" s="7" t="inlineStr">
         <is>
-          <t>HAVAL</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G99" s="6" t="n">
@@ -21767,17 +21687,17 @@
       </c>
       <c r="B100" s="11" t="inlineStr">
         <is>
-          <t>Моторленд (Воронеж)</t>
+          <t>Петровский</t>
         </is>
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>Моторленд</t>
+          <t>Петровский</t>
         </is>
       </c>
       <c r="D100" s="8" t="inlineStr">
         <is>
-          <t>3662259794</t>
+          <t>7813382729</t>
         </is>
       </c>
       <c r="E100" s="11" t="inlineStr">
@@ -21787,7 +21707,7 @@
       </c>
       <c r="F100" s="11" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>OMODA</t>
         </is>
       </c>
       <c r="G100" s="10" t="n">
@@ -21821,17 +21741,17 @@
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>7813382729</t>
+          <t>7718752313</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>Санкт-Петербург</t>
+          <t>Москва</t>
         </is>
       </c>
       <c r="F101" s="7" t="inlineStr">
         <is>
-          <t>OMODA</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G101" s="6" t="n">
@@ -21863,19 +21783,15 @@
           <t>Петровский</t>
         </is>
       </c>
-      <c r="D102" s="8" t="inlineStr">
-        <is>
-          <t>7718752313</t>
-        </is>
-      </c>
+      <c r="D102" s="8" t="inlineStr"/>
       <c r="E102" s="11" t="inlineStr">
         <is>
-          <t>Москва</t>
+          <t>Санкт-Петербург</t>
         </is>
       </c>
       <c r="F102" s="11" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>МОСКВИЧ</t>
         </is>
       </c>
       <c r="G102" s="10" t="n">
@@ -21899,23 +21815,27 @@
       </c>
       <c r="B103" s="7" t="inlineStr">
         <is>
-          <t>Петровский</t>
+          <t>Прагматика</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>Петровский</t>
-        </is>
-      </c>
-      <c r="D103" s="4" t="inlineStr"/>
+          <t>Прагматика Великие Луки</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>6027196721</t>
+        </is>
+      </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>Санкт-Петербург</t>
+          <t>Великие Луки</t>
         </is>
       </c>
       <c r="F103" s="7" t="inlineStr">
         <is>
-          <t>МОСКВИЧ</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G103" s="6" t="n">
@@ -21944,17 +21864,17 @@
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>Прагматика Великие Луки</t>
+          <t>Прагматика Великий Новгород</t>
         </is>
       </c>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>6027196721</t>
+          <t>5321198672</t>
         </is>
       </c>
       <c r="E104" s="11" t="inlineStr">
         <is>
-          <t>Великие Луки</t>
+          <t>Великий Новгород</t>
         </is>
       </c>
       <c r="F104" s="11" t="inlineStr">
@@ -21988,17 +21908,17 @@
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>Прагматика Великий Новгород</t>
+          <t>Прагматика Мурманск</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>5321198672</t>
+          <t>5190098569</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>Великий Новгород</t>
+          <t>Мурманск</t>
         </is>
       </c>
       <c r="F105" s="7" t="inlineStr">
@@ -22032,17 +21952,17 @@
       </c>
       <c r="C106" s="11" t="inlineStr">
         <is>
-          <t>Прагматика Мурманск</t>
+          <t>Прагматика Петрозаводск</t>
         </is>
       </c>
       <c r="D106" s="8" t="inlineStr">
         <is>
-          <t>5190098569</t>
+          <t>1001340114</t>
         </is>
       </c>
       <c r="E106" s="11" t="inlineStr">
         <is>
-          <t>Мурманск</t>
+          <t>Петрозаводск</t>
         </is>
       </c>
       <c r="F106" s="11" t="inlineStr">
@@ -22076,17 +21996,17 @@
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>Прагматика Петрозаводск</t>
+          <t>Прагматика</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>1001340114</t>
+          <t>6027196721</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>Петрозаводск</t>
+          <t>Псков</t>
         </is>
       </c>
       <c r="F107" s="7" t="inlineStr">
@@ -22120,17 +22040,17 @@
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>Прагматика</t>
+          <t>Прагматика Автоцентр Парнас</t>
         </is>
       </c>
       <c r="D108" s="8" t="inlineStr">
         <is>
-          <t>6027196721</t>
+          <t>7802914957</t>
         </is>
       </c>
       <c r="E108" s="11" t="inlineStr">
         <is>
-          <t>Псков</t>
+          <t>Санкт-Петербург</t>
         </is>
       </c>
       <c r="F108" s="11" t="inlineStr">
@@ -22164,12 +22084,12 @@
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>Прагматика Автоцентр Парнас</t>
+          <t>Прагматика Лада Купчино</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>7802914957</t>
+          <t>7816716659</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
@@ -22208,12 +22128,12 @@
       </c>
       <c r="C110" s="11" t="inlineStr">
         <is>
-          <t>Прагматика Лада Купчино</t>
+          <t>Прагматика ВО</t>
         </is>
       </c>
       <c r="D110" s="8" t="inlineStr">
         <is>
-          <t>7816716659</t>
+          <t>7801288506</t>
         </is>
       </c>
       <c r="E110" s="11" t="inlineStr">
@@ -22247,27 +22167,23 @@
       </c>
       <c r="B111" s="7" t="inlineStr">
         <is>
-          <t>Прагматика</t>
+          <t>Прагматика пилот (ФДЦ) новые</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>Прагматика ВО</t>
-        </is>
-      </c>
-      <c r="D111" s="4" t="inlineStr">
-        <is>
-          <t>7801288506</t>
-        </is>
-      </c>
+          <t>Прагматика пилот (ФДЦ) новые</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr"/>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>Санкт-Петербург</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F111" s="7" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>CHANGAN</t>
         </is>
       </c>
       <c r="G111" s="6" t="n">
@@ -22281,7 +22197,7 @@
       </c>
       <c r="J111" s="7" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -22291,12 +22207,12 @@
       </c>
       <c r="B112" s="11" t="inlineStr">
         <is>
-          <t>Прагматика пилот (ФДЦ) новые</t>
+          <t>Приоритет_Прагматика пилот ФДЦ</t>
         </is>
       </c>
       <c r="C112" s="11" t="inlineStr">
         <is>
-          <t>Прагматика пилот (ФДЦ) новые</t>
+          <t>Приоритет_Прагматика пилот ФДЦ</t>
         </is>
       </c>
       <c r="D112" s="8" t="inlineStr"/>
@@ -22307,7 +22223,7 @@
       </c>
       <c r="F112" s="11" t="inlineStr">
         <is>
-          <t>CHANGAN</t>
+          <t>FORD</t>
         </is>
       </c>
       <c r="G112" s="10" t="n">
@@ -22331,12 +22247,12 @@
       </c>
       <c r="B113" s="7" t="inlineStr">
         <is>
-          <t>Приоритет_Прагматика пилот ФДЦ</t>
+          <t>Приоритет_Сигма СПб</t>
         </is>
       </c>
       <c r="C113" s="7" t="inlineStr">
         <is>
-          <t>Приоритет_Прагматика пилот ФДЦ</t>
+          <t>Приоритет_Сигма СПб</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr"/>
@@ -22347,7 +22263,7 @@
       </c>
       <c r="F113" s="7" t="inlineStr">
         <is>
-          <t>FORD</t>
+          <t>HAVAL</t>
         </is>
       </c>
       <c r="G113" s="6" t="n">
@@ -22371,12 +22287,12 @@
       </c>
       <c r="B114" s="11" t="inlineStr">
         <is>
-          <t>Приоритет_Сигма СПб</t>
+          <t>Р-Моторс Лада (ОП Барнаул)</t>
         </is>
       </c>
       <c r="C114" s="11" t="inlineStr">
         <is>
-          <t>Приоритет_Сигма СПб</t>
+          <t>ONLINE Р-Моторс Лада (ОП Барнаул)</t>
         </is>
       </c>
       <c r="D114" s="8" t="inlineStr"/>
@@ -22387,7 +22303,7 @@
       </c>
       <c r="F114" s="11" t="inlineStr">
         <is>
-          <t>HAVAL</t>
+          <t>Новые авто</t>
         </is>
       </c>
       <c r="G114" s="10" t="n">
@@ -22411,23 +22327,27 @@
       </c>
       <c r="B115" s="7" t="inlineStr">
         <is>
-          <t>Р-Моторс Лада (ОП Барнаул)</t>
+          <t>РГС</t>
         </is>
       </c>
       <c r="C115" s="7" t="inlineStr">
         <is>
-          <t>ONLINE Р-Моторс Лада (ОП Барнаул)</t>
-        </is>
-      </c>
-      <c r="D115" s="4" t="inlineStr"/>
+          <t>РГС</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>2904030348</t>
+        </is>
+      </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Котлас</t>
         </is>
       </c>
       <c r="F115" s="7" t="inlineStr">
         <is>
-          <t>Новые авто</t>
+          <t>SOLARIS</t>
         </is>
       </c>
       <c r="G115" s="6" t="n">
@@ -22441,7 +22361,7 @@
       </c>
       <c r="J115" s="7" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -22451,27 +22371,27 @@
       </c>
       <c r="B116" s="11" t="inlineStr">
         <is>
-          <t>РГС</t>
+          <t>СВ-Авто</t>
         </is>
       </c>
       <c r="C116" s="11" t="inlineStr">
         <is>
-          <t>РГС</t>
+          <t>СВ-Авто</t>
         </is>
       </c>
       <c r="D116" s="8" t="inlineStr">
         <is>
-          <t>2904030348</t>
+          <t>4205206560</t>
         </is>
       </c>
       <c r="E116" s="11" t="inlineStr">
         <is>
-          <t>Котлас</t>
+          <t>Новокузнецк</t>
         </is>
       </c>
       <c r="F116" s="11" t="inlineStr">
         <is>
-          <t>SOLARIS</t>
+          <t>CHERY</t>
         </is>
       </c>
       <c r="G116" s="10" t="n">
@@ -22495,27 +22415,27 @@
       </c>
       <c r="B117" s="7" t="inlineStr">
         <is>
-          <t>СВ-Авто</t>
+          <t>ТЮМЕНЬ-АВТОВАЗ (АО "ТЮМЕНЬ-АВТОВАЗ")</t>
         </is>
       </c>
       <c r="C117" s="7" t="inlineStr">
         <is>
-          <t>СВ-Авто</t>
+          <t>Тюмень-Автоваз</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>4205206560</t>
+          <t>7203083968</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>Новокузнецк</t>
+          <t>Тюмень</t>
         </is>
       </c>
       <c r="F117" s="7" t="inlineStr">
         <is>
-          <t>CHERY</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G117" s="6" t="n">
@@ -22539,27 +22459,27 @@
       </c>
       <c r="B118" s="11" t="inlineStr">
         <is>
-          <t>ТЮМЕНЬ-АВТОВАЗ (АО "ТЮМЕНЬ-АВТОВАЗ")</t>
+          <t>Фастар</t>
         </is>
       </c>
       <c r="C118" s="11" t="inlineStr">
         <is>
-          <t>Тюмень-Автоваз</t>
+          <t>Фастар</t>
         </is>
       </c>
       <c r="D118" s="8" t="inlineStr">
         <is>
-          <t>7203083968</t>
+          <t>5404062153</t>
         </is>
       </c>
       <c r="E118" s="11" t="inlineStr">
         <is>
-          <t>Тюмень</t>
+          <t>Новосибирск</t>
         </is>
       </c>
       <c r="F118" s="11" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>BELGEE</t>
         </is>
       </c>
       <c r="G118" s="10" t="n">
@@ -22583,27 +22503,23 @@
       </c>
       <c r="B119" s="7" t="inlineStr">
         <is>
-          <t>Фастар</t>
+          <t>ФДЦ Алгоритм Сервис Лада</t>
         </is>
       </c>
       <c r="C119" s="7" t="inlineStr">
         <is>
-          <t>Фастар</t>
-        </is>
-      </c>
-      <c r="D119" s="4" t="inlineStr">
-        <is>
-          <t>5404062153</t>
-        </is>
-      </c>
+          <t>ONLINE ФДЦ Алгоритм Сервис Лада</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr"/>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>Новосибирск</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F119" s="7" t="inlineStr">
         <is>
-          <t>BELGEE</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G119" s="6" t="n">
@@ -22617,7 +22533,7 @@
       </c>
       <c r="J119" s="7" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -22627,23 +22543,27 @@
       </c>
       <c r="B120" s="11" t="inlineStr">
         <is>
-          <t>ФДЦ Алгоритм Сервис Лада</t>
+          <t>ЧЕРИ ЦЕНТР ДИНАМИКА АРХАНГЕЛЬСК ОНЛАЙН</t>
         </is>
       </c>
       <c r="C120" s="11" t="inlineStr">
         <is>
-          <t>ONLINE ФДЦ Алгоритм Сервис Лада</t>
-        </is>
-      </c>
-      <c r="D120" s="8" t="inlineStr"/>
+          <t>ЧЕРИ ЦЕНТР ДИНАМИКА АРХАНГЕЛЬСК ОНЛАЙН</t>
+        </is>
+      </c>
+      <c r="D120" s="8" t="inlineStr">
+        <is>
+          <t>1101096766</t>
+        </is>
+      </c>
       <c r="E120" s="11" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Архангельск</t>
         </is>
       </c>
       <c r="F120" s="11" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>CHERY</t>
         </is>
       </c>
       <c r="G120" s="10" t="n">
@@ -22657,7 +22577,7 @@
       </c>
       <c r="J120" s="11" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -22667,22 +22587,22 @@
       </c>
       <c r="B121" s="7" t="inlineStr">
         <is>
-          <t>ЧЕРИ ЦЕНТР ДИНАМИКА АРХАНГЕЛЬСК ОНЛАЙН</t>
+          <t>ЧЕРИ ЦЕНТР СИГМА ОНЛАЙН</t>
         </is>
       </c>
       <c r="C121" s="7" t="inlineStr">
         <is>
-          <t>ЧЕРИ ЦЕНТР ДИНАМИКА АРХАНГЕЛЬСК ОНЛАЙН</t>
+          <t>ЧЕРИ ЦЕНТР СИГМА ОНЛАЙН</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>1101096766</t>
+          <t>7813649997</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>Архангельск</t>
+          <t>Санкт-Петербург</t>
         </is>
       </c>
       <c r="F121" s="7" t="inlineStr">
@@ -22711,22 +22631,22 @@
       </c>
       <c r="B122" s="11" t="inlineStr">
         <is>
-          <t>ЧЕРИ ЦЕНТР СИГМА ОНЛАЙН</t>
+          <t>Чери Центр Форвард-Авто</t>
         </is>
       </c>
       <c r="C122" s="11" t="inlineStr">
         <is>
-          <t>ЧЕРИ ЦЕНТР СИГМА ОНЛАЙН</t>
+          <t>Чери Центр Форвард-Авто</t>
         </is>
       </c>
       <c r="D122" s="8" t="inlineStr">
         <is>
-          <t>7813649997</t>
+          <t>5906145075</t>
         </is>
       </c>
       <c r="E122" s="11" t="inlineStr">
         <is>
-          <t>Санкт-Петербург</t>
+          <t>Тюмень</t>
         </is>
       </c>
       <c r="F122" s="11" t="inlineStr">
@@ -28731,7 +28651,7 @@
       </c>
       <c r="C132" s="17" t="inlineStr">
         <is>
-          <t>ONLINE ООО "АВТОСФЕРА", СберАвто</t>
+          <t>СберАвто, ONLINE ООО "АВТОСФЕРА"</t>
         </is>
       </c>
       <c r="D132" s="16" t="inlineStr"/>

</xml_diff>

<commit_message>
fix(kam): ensure full Avtomir allocation to Kuznetsov except Simferopol to Soldatova
</commit_message>
<xml_diff>
--- a/Закрепление_партнеров_по_КАМ_Сентябрь_2026.xlsx
+++ b/Закрепление_партнеров_по_КАМ_Сентябрь_2026.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Валерия Солдатова" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Андрей Кузнецов'!$A$4:$J$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Андрей Кузнецов'!$A$4:$J$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Алексей Чихарев'!$A$4:$J$214</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Евгения Добролюбова'!$A$4:$J$100</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Светлана Дариенко'!$A$4:$J$128</definedName>
@@ -613,16 +613,16 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>196</v>
+        <v>255</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>196</v>
+        <v>255</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -670,13 +670,13 @@
         <v>96</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>154</v>
+        <v>95</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>154</v>
+        <v>95</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="D10" s="14" t="n">
         <v>771</v>
@@ -770,7 +770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J74"/>
+  <dimension ref="A1:J77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -795,7 +795,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Всего объектов в портфеле: 69 ДЦ. Источник: OEM СберАвто финал (15)</t>
+          <t>Всего объектов в портфеле: 72 ДЦ. Источник: OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -1342,41 +1342,37 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>РОЛЬФ</t>
+          <t>ФДЦ Автосеть АМК РФ</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>ГК Рольф</t>
-        </is>
-      </c>
-      <c r="D16" s="16" t="inlineStr">
-        <is>
-          <t>5047254063</t>
-        </is>
-      </c>
+          <t>ONLINE ООО "АМКАПИТАЛ"</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr"/>
       <c r="E16" s="17" t="inlineStr">
         <is>
-          <t>Москва</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F16" s="17" t="inlineStr">
         <is>
-          <t>OMODA</t>
+          <t>CHANGAN, JETOUR, GAC</t>
         </is>
       </c>
       <c r="G16" s="18" t="n">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="H16" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I16" s="18" t="n">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -1445,7 +1441,7 @@
       </c>
       <c r="E18" s="17" t="inlineStr">
         <is>
-          <t>Санкт-Петербург</t>
+          <t>Москва</t>
         </is>
       </c>
       <c r="F18" s="17" t="inlineStr">
@@ -1479,7 +1475,7 @@
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
-          <t>Рольф Алтуфьево</t>
+          <t>ГК Рольф</t>
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr">
@@ -1489,12 +1485,12 @@
       </c>
       <c r="E19" s="17" t="inlineStr">
         <is>
-          <t>Москва</t>
+          <t>Санкт-Петербург</t>
         </is>
       </c>
       <c r="F19" s="17" t="inlineStr">
         <is>
-          <t>GEELY</t>
+          <t>OMODA</t>
         </is>
       </c>
       <c r="G19" s="18" t="n">
@@ -1523,7 +1519,7 @@
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>Рольф ЮГ  Haval PRO</t>
+          <t>Рольф Алтуфьево</t>
         </is>
       </c>
       <c r="D20" s="16" t="inlineStr">
@@ -1538,7 +1534,7 @@
       </c>
       <c r="F20" s="17" t="inlineStr">
         <is>
-          <t>HAVAL</t>
+          <t>GEELY</t>
         </is>
       </c>
       <c r="G20" s="18" t="n">
@@ -1567,7 +1563,7 @@
       </c>
       <c r="C21" s="17" t="inlineStr">
         <is>
-          <t>Рольф</t>
+          <t>Рольф ЮГ  Haval PRO</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr">
@@ -1582,7 +1578,7 @@
       </c>
       <c r="F21" s="17" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>HAVAL</t>
         </is>
       </c>
       <c r="G21" s="18" t="n">
@@ -1611,7 +1607,7 @@
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>РОЛЬФ</t>
+          <t>Рольф</t>
         </is>
       </c>
       <c r="D22" s="16" t="inlineStr">
@@ -1626,7 +1622,7 @@
       </c>
       <c r="F22" s="17" t="inlineStr">
         <is>
-          <t>SOLARIS</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G22" s="18" t="n">
@@ -1655,7 +1651,7 @@
       </c>
       <c r="C23" s="17" t="inlineStr">
         <is>
-          <t>Рольф Алтуфьево</t>
+          <t>РОЛЬФ</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
@@ -1670,7 +1666,7 @@
       </c>
       <c r="F23" s="17" t="inlineStr">
         <is>
-          <t>Hyundai</t>
+          <t>SOLARIS</t>
         </is>
       </c>
       <c r="G23" s="18" t="n">
@@ -1699,7 +1695,7 @@
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>Рольф Сити</t>
+          <t>Рольф Алтуфьево</t>
         </is>
       </c>
       <c r="D24" s="16" t="inlineStr">
@@ -1714,7 +1710,7 @@
       </c>
       <c r="F24" s="17" t="inlineStr">
         <is>
-          <t>РОЛЬФ ИМПОРТ</t>
+          <t>Hyundai</t>
         </is>
       </c>
       <c r="G24" s="18" t="n">
@@ -1743,7 +1739,7 @@
       </c>
       <c r="C25" s="17" t="inlineStr">
         <is>
-          <t>Рольф Химки</t>
+          <t>Рольф Сити</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr">
@@ -1787,7 +1783,7 @@
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>Рольф ЮГ</t>
+          <t>Рольф Химки</t>
         </is>
       </c>
       <c r="D26" s="16" t="inlineStr">
@@ -1831,7 +1827,7 @@
       </c>
       <c r="C27" s="17" t="inlineStr">
         <is>
-          <t>Рольф Восток</t>
+          <t>Рольф ЮГ</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -1846,7 +1842,7 @@
       </c>
       <c r="F27" s="17" t="inlineStr">
         <is>
-          <t>Mazda</t>
+          <t>РОЛЬФ ИМПОРТ</t>
         </is>
       </c>
       <c r="G27" s="18" t="n">
@@ -1875,7 +1871,7 @@
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>Рольф Химки</t>
+          <t>Рольф Восток</t>
         </is>
       </c>
       <c r="D28" s="16" t="inlineStr">
@@ -1890,7 +1886,7 @@
       </c>
       <c r="F28" s="17" t="inlineStr">
         <is>
-          <t>РОЛЬФ ИМПОРТ</t>
+          <t>Mazda</t>
         </is>
       </c>
       <c r="G28" s="18" t="n">
@@ -1919,7 +1915,7 @@
       </c>
       <c r="C29" s="17" t="inlineStr">
         <is>
-          <t>Рольф ЮГ</t>
+          <t>Рольф Химки</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -1963,7 +1959,7 @@
       </c>
       <c r="C30" s="17" t="inlineStr">
         <is>
-          <t>Рольф Волгоградский</t>
+          <t>Рольф ЮГ</t>
         </is>
       </c>
       <c r="D30" s="16" t="inlineStr">
@@ -1978,7 +1974,7 @@
       </c>
       <c r="F30" s="17" t="inlineStr">
         <is>
-          <t>Toyota</t>
+          <t>РОЛЬФ ИМПОРТ</t>
         </is>
       </c>
       <c r="G30" s="18" t="n">
@@ -2007,7 +2003,7 @@
       </c>
       <c r="C31" s="17" t="inlineStr">
         <is>
-          <t>Рольф Сити</t>
+          <t>Рольф Волгоградский</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -2022,7 +2018,7 @@
       </c>
       <c r="F31" s="17" t="inlineStr">
         <is>
-          <t>РОЛЬФ ИМПОРТ</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="G31" s="18" t="n">
@@ -2051,7 +2047,7 @@
       </c>
       <c r="C32" s="17" t="inlineStr">
         <is>
-          <t>Рольф Химки</t>
+          <t>Рольф Сити</t>
         </is>
       </c>
       <c r="D32" s="16" t="inlineStr">
@@ -2095,7 +2091,7 @@
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
-          <t>Рольф Центр</t>
+          <t>Рольф Химки</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -2139,7 +2135,7 @@
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>Рольф Ясенево</t>
+          <t>Рольф Центр</t>
         </is>
       </c>
       <c r="D34" s="16" t="inlineStr">
@@ -2183,7 +2179,7 @@
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
-          <t>Рольф Вешки</t>
+          <t>Рольф Ясенево</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
@@ -2198,7 +2194,7 @@
       </c>
       <c r="F35" s="17" t="inlineStr">
         <is>
-          <t>Volkswagen</t>
+          <t>РОЛЬФ ИМПОРТ</t>
         </is>
       </c>
       <c r="G35" s="18" t="n">
@@ -2227,7 +2223,7 @@
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>Рольф Центр</t>
+          <t>Рольф Вешки</t>
         </is>
       </c>
       <c r="D36" s="16" t="inlineStr">
@@ -2242,7 +2238,7 @@
       </c>
       <c r="F36" s="17" t="inlineStr">
         <is>
-          <t>РОЛЬФ ИМПОРТ</t>
+          <t>Volkswagen</t>
         </is>
       </c>
       <c r="G36" s="18" t="n">
@@ -2271,7 +2267,7 @@
       </c>
       <c r="C37" s="17" t="inlineStr">
         <is>
-          <t>Рольф ЮГ</t>
+          <t>Рольф Центр</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
@@ -2310,37 +2306,37 @@
       </c>
       <c r="B38" s="17" t="inlineStr">
         <is>
-          <t>ГК АГАТ</t>
+          <t>РОЛЬФ</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
-          <t>ГК Агат</t>
+          <t>Рольф ЮГ</t>
         </is>
       </c>
       <c r="D38" s="16" t="inlineStr">
         <is>
-          <t>3459070992</t>
+          <t>5047254063</t>
         </is>
       </c>
       <c r="E38" s="17" t="inlineStr">
         <is>
-          <t>Волгоград</t>
+          <t>Москва</t>
         </is>
       </c>
       <c r="F38" s="17" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>РОЛЬФ ИМПОРТ</t>
         </is>
       </c>
       <c r="G38" s="18" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="H38" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I38" s="18" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="J38" s="17" t="inlineStr">
         <is>
@@ -2364,7 +2360,7 @@
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>3443067465</t>
+          <t>3459070992</t>
         </is>
       </c>
       <c r="E39" s="17" t="inlineStr">
@@ -2403,17 +2399,17 @@
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>ГК АГАТ Лада</t>
+          <t>ГК Агат</t>
         </is>
       </c>
       <c r="D40" s="16" t="inlineStr">
         <is>
-          <t>5261037364</t>
+          <t>3443067465</t>
         </is>
       </c>
       <c r="E40" s="17" t="inlineStr">
         <is>
-          <t>Нижний Новгород</t>
+          <t>Волгоград</t>
         </is>
       </c>
       <c r="F40" s="17" t="inlineStr">
@@ -2452,7 +2448,7 @@
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>5257188868</t>
+          <t>5261037364</t>
         </is>
       </c>
       <c r="E41" s="17" t="inlineStr">
@@ -2491,13 +2487,17 @@
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>ГК Агат</t>
-        </is>
-      </c>
-      <c r="D42" s="16" t="inlineStr"/>
+          <t>ГК АГАТ Лада</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>5257188868</t>
+        </is>
+      </c>
       <c r="E42" s="17" t="inlineStr">
         <is>
-          <t>Саратов</t>
+          <t>Нижний Новгород</t>
         </is>
       </c>
       <c r="F42" s="17" t="inlineStr">
@@ -2537,7 +2537,7 @@
       <c r="D43" s="16" t="inlineStr"/>
       <c r="E43" s="17" t="inlineStr">
         <is>
-          <t>Сыктывкар</t>
+          <t>Саратов</t>
         </is>
       </c>
       <c r="F43" s="17" t="inlineStr">
@@ -2574,19 +2574,15 @@
           <t>ГК Агат</t>
         </is>
       </c>
-      <c r="D44" s="16" t="inlineStr">
-        <is>
-          <t>3443092790</t>
-        </is>
-      </c>
+      <c r="D44" s="16" t="inlineStr"/>
       <c r="E44" s="17" t="inlineStr">
         <is>
-          <t>Волгоград</t>
+          <t>Сыктывкар</t>
         </is>
       </c>
       <c r="F44" s="17" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G44" s="18" t="n">
@@ -2615,17 +2611,17 @@
       </c>
       <c r="C45" s="17" t="inlineStr">
         <is>
-          <t>АГАТ</t>
+          <t>ГК Агат</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>5257100888</t>
+          <t>3443092790</t>
         </is>
       </c>
       <c r="E45" s="17" t="inlineStr">
         <is>
-          <t>Нижний Новгород</t>
+          <t>Волгоград</t>
         </is>
       </c>
       <c r="F45" s="17" t="inlineStr">
@@ -2664,7 +2660,7 @@
       </c>
       <c r="D46" s="16" t="inlineStr">
         <is>
-          <t>5258089355</t>
+          <t>5257100888</t>
         </is>
       </c>
       <c r="E46" s="17" t="inlineStr">
@@ -2708,12 +2704,12 @@
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>5257188836</t>
+          <t>5258089355</t>
         </is>
       </c>
       <c r="E47" s="17" t="inlineStr">
         <is>
-          <t>Саранск</t>
+          <t>Нижний Новгород</t>
         </is>
       </c>
       <c r="F47" s="17" t="inlineStr">
@@ -2747,17 +2743,17 @@
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>ГК АГАТ</t>
+          <t>АГАТ</t>
         </is>
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>5257208916</t>
+          <t>5257188836</t>
         </is>
       </c>
       <c r="E48" s="17" t="inlineStr">
         <is>
-          <t>Ярославль</t>
+          <t>Саранск</t>
         </is>
       </c>
       <c r="F48" s="17" t="inlineStr">
@@ -2786,37 +2782,41 @@
       </c>
       <c r="B49" s="17" t="inlineStr">
         <is>
-          <t>ГК КОРС Джетур</t>
+          <t>ГК АГАТ</t>
         </is>
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>ООО "КОРС НОВОМОСКОВСК" ONLINE</t>
-        </is>
-      </c>
-      <c r="D49" s="16" t="inlineStr"/>
+          <t>ГК АГАТ</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>5257208916</t>
+        </is>
+      </c>
       <c r="E49" s="17" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Ярославль</t>
         </is>
       </c>
       <c r="F49" s="17" t="inlineStr">
         <is>
-          <t>GAC, SOUEAST, JETOUR</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G49" s="18" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="H49" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I49" s="18" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="J49" s="17" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -2826,41 +2826,37 @@
       </c>
       <c r="B50" s="17" t="inlineStr">
         <is>
-          <t>Fresh Auto</t>
+          <t>ГК КОРС Джетур</t>
         </is>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>Фреш</t>
-        </is>
-      </c>
-      <c r="D50" s="16" t="inlineStr">
-        <is>
-          <t>9723038901</t>
-        </is>
-      </c>
+          <t>ООО "КОРС НОВОМОСКОВСК" ONLINE</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr"/>
       <c r="E50" s="17" t="inlineStr">
         <is>
-          <t>Воронеж</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F50" s="17" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>SOUEAST, JETOUR, GAC</t>
         </is>
       </c>
       <c r="G50" s="18" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="H50" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I50" s="18" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="J50" s="17" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2881,7 @@
       </c>
       <c r="E51" s="17" t="inlineStr">
         <is>
-          <t>Ростов-на-Дону</t>
+          <t>Воронеж</t>
         </is>
       </c>
       <c r="F51" s="17" t="inlineStr">
@@ -2914,27 +2910,27 @@
       </c>
       <c r="B52" s="17" t="inlineStr">
         <is>
-          <t>ГК Автомир</t>
+          <t>Fresh Auto</t>
         </is>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
-          <t>ГК АВТОМИР</t>
+          <t>Фреш</t>
         </is>
       </c>
       <c r="D52" s="16" t="inlineStr">
         <is>
-          <t>7708607959</t>
+          <t>9723038901</t>
         </is>
       </c>
       <c r="E52" s="17" t="inlineStr">
         <is>
-          <t>Москва</t>
+          <t>Ростов-на-Дону</t>
         </is>
       </c>
       <c r="F52" s="17" t="inlineStr">
         <is>
-          <t>GEELY</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G52" s="18" t="n">
@@ -2963,22 +2959,22 @@
       </c>
       <c r="C53" s="17" t="inlineStr">
         <is>
-          <t>ГК Автомир</t>
+          <t>ГК АВТОМИР</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>7730568529</t>
+          <t>7708607959</t>
         </is>
       </c>
       <c r="E53" s="17" t="inlineStr">
         <is>
-          <t>Брянск</t>
+          <t>Москва</t>
         </is>
       </c>
       <c r="F53" s="17" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>GEELY,BELGEE</t>
         </is>
       </c>
       <c r="G53" s="18" t="n">
@@ -3007,22 +3003,22 @@
       </c>
       <c r="C54" s="17" t="inlineStr">
         <is>
-          <t>ГК Автомир</t>
+          <t>ГК АВТОМИР</t>
         </is>
       </c>
       <c r="D54" s="16" t="inlineStr">
         <is>
-          <t>7730568529</t>
+          <t>7708607959</t>
         </is>
       </c>
       <c r="E54" s="17" t="inlineStr">
         <is>
-          <t>Ярославль</t>
+          <t>Москва</t>
         </is>
       </c>
       <c r="F54" s="17" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>GEELY</t>
         </is>
       </c>
       <c r="G54" s="18" t="n">
@@ -3051,7 +3047,7 @@
       </c>
       <c r="C55" s="17" t="inlineStr">
         <is>
-          <t>ГК Автомир</t>
+          <t>ГК АВТОМИР</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
@@ -3066,7 +3062,7 @@
       </c>
       <c r="F55" s="17" t="inlineStr">
         <is>
-          <t>HAVAL</t>
+          <t>GEELY,BELGEE</t>
         </is>
       </c>
       <c r="G55" s="18" t="n">
@@ -3095,22 +3091,22 @@
       </c>
       <c r="C56" s="17" t="inlineStr">
         <is>
-          <t>Автомир</t>
+          <t>ГК Автомир</t>
         </is>
       </c>
       <c r="D56" s="16" t="inlineStr">
         <is>
-          <t>7708607959</t>
+          <t>7730568529</t>
         </is>
       </c>
       <c r="E56" s="17" t="inlineStr">
         <is>
-          <t>Москва</t>
+          <t>Брянск</t>
         </is>
       </c>
       <c r="F56" s="17" t="inlineStr">
         <is>
-          <t>CHANGAN</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G56" s="18" t="n">
@@ -3139,22 +3135,22 @@
       </c>
       <c r="C57" s="17" t="inlineStr">
         <is>
-          <t>Автомир</t>
+          <t>ГК Автомир</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>7708607959</t>
+          <t>7730568529</t>
         </is>
       </c>
       <c r="E57" s="17" t="inlineStr">
         <is>
-          <t>Москва</t>
+          <t>Ярославль</t>
         </is>
       </c>
       <c r="F57" s="17" t="inlineStr">
         <is>
-          <t>CHANGAN</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G57" s="18" t="n">
@@ -3193,12 +3189,12 @@
       </c>
       <c r="E58" s="17" t="inlineStr">
         <is>
-          <t>Санкт-Петербург</t>
+          <t>Москва</t>
         </is>
       </c>
       <c r="F58" s="17" t="inlineStr">
         <is>
-          <t>CHANGAN</t>
+          <t>HAVAL</t>
         </is>
       </c>
       <c r="G58" s="18" t="n">
@@ -3242,7 +3238,7 @@
       </c>
       <c r="F59" s="17" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>CHANGAN</t>
         </is>
       </c>
       <c r="G59" s="18" t="n">
@@ -3286,7 +3282,7 @@
       </c>
       <c r="F60" s="17" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>CHANGAN</t>
         </is>
       </c>
       <c r="G60" s="18" t="n">
@@ -3315,22 +3311,22 @@
       </c>
       <c r="C61" s="17" t="inlineStr">
         <is>
-          <t>ГК АВТОМИР</t>
+          <t>ГК Автомир</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>7730569353</t>
+          <t>7708607959</t>
         </is>
       </c>
       <c r="E61" s="17" t="inlineStr">
         <is>
-          <t>Москва</t>
+          <t>Санкт-Петербург</t>
         </is>
       </c>
       <c r="F61" s="17" t="inlineStr">
         <is>
-          <t>SOLARIS</t>
+          <t>CHANGAN</t>
         </is>
       </c>
       <c r="G61" s="18" t="n">
@@ -3359,12 +3355,12 @@
       </c>
       <c r="C62" s="17" t="inlineStr">
         <is>
-          <t>ГК АВТОМИР</t>
+          <t>Автомир</t>
         </is>
       </c>
       <c r="D62" s="16" t="inlineStr">
         <is>
-          <t>7730569353</t>
+          <t>7708607959</t>
         </is>
       </c>
       <c r="E62" s="17" t="inlineStr">
@@ -3374,7 +3370,7 @@
       </c>
       <c r="F62" s="17" t="inlineStr">
         <is>
-          <t>SOLARIS</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G62" s="18" t="n">
@@ -3393,130 +3389,134 @@
       </c>
     </row>
     <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="4" t="n">
+      <c r="A63" s="16" t="n">
         <v>59</v>
       </c>
-      <c r="B63" s="7" t="inlineStr">
-        <is>
-          <t>Fresh Haval мин воды</t>
-        </is>
-      </c>
-      <c r="C63" s="7" t="inlineStr">
-        <is>
-          <t>Fresh Haval мин воды</t>
-        </is>
-      </c>
-      <c r="D63" s="4" t="inlineStr">
-        <is>
-          <t>3443137377</t>
-        </is>
-      </c>
-      <c r="E63" s="7" t="inlineStr">
-        <is>
-          <t>Минеральные Воды</t>
-        </is>
-      </c>
-      <c r="F63" s="7" t="inlineStr">
-        <is>
-          <t>HAVAL</t>
-        </is>
-      </c>
-      <c r="G63" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H63" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I63" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J63" s="7" t="inlineStr">
+      <c r="B63" s="17" t="inlineStr">
+        <is>
+          <t>ГК Автомир</t>
+        </is>
+      </c>
+      <c r="C63" s="17" t="inlineStr">
+        <is>
+          <t>Автомир</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>7708607959</t>
+        </is>
+      </c>
+      <c r="E63" s="17" t="inlineStr">
+        <is>
+          <t>Москва</t>
+        </is>
+      </c>
+      <c r="F63" s="17" t="inlineStr">
+        <is>
+          <t>JETOUR</t>
+        </is>
+      </c>
+      <c r="G63" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="H63" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="J63" s="17" t="inlineStr">
         <is>
           <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
     <row r="64" ht="20" customHeight="1">
-      <c r="A64" s="8" t="n">
+      <c r="A64" s="16" t="n">
         <v>60</v>
       </c>
-      <c r="B64" s="11" t="inlineStr">
-        <is>
-          <t>Fresh Haval Ростов</t>
-        </is>
-      </c>
-      <c r="C64" s="11" t="inlineStr">
-        <is>
-          <t>Fresh Haval Ростов</t>
-        </is>
-      </c>
-      <c r="D64" s="8" t="inlineStr">
-        <is>
-          <t>3443137377</t>
-        </is>
-      </c>
-      <c r="E64" s="11" t="inlineStr">
-        <is>
-          <t>Ростов-на-Дону</t>
-        </is>
-      </c>
-      <c r="F64" s="11" t="inlineStr">
-        <is>
-          <t>HAVAL</t>
-        </is>
-      </c>
-      <c r="G64" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H64" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I64" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J64" s="11" t="inlineStr">
+      <c r="B64" s="17" t="inlineStr">
+        <is>
+          <t>ГК Автомир</t>
+        </is>
+      </c>
+      <c r="C64" s="17" t="inlineStr">
+        <is>
+          <t>ГК АВТОМИР</t>
+        </is>
+      </c>
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>7730569353</t>
+        </is>
+      </c>
+      <c r="E64" s="17" t="inlineStr">
+        <is>
+          <t>Москва</t>
+        </is>
+      </c>
+      <c r="F64" s="17" t="inlineStr">
+        <is>
+          <t>SOLARIS</t>
+        </is>
+      </c>
+      <c r="G64" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="H64" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="J64" s="17" t="inlineStr">
         <is>
           <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
     <row r="65" ht="20" customHeight="1">
-      <c r="A65" s="4" t="n">
+      <c r="A65" s="16" t="n">
         <v>61</v>
       </c>
-      <c r="B65" s="7" t="inlineStr">
-        <is>
-          <t>Team63Auto</t>
-        </is>
-      </c>
-      <c r="C65" s="7" t="inlineStr">
-        <is>
-          <t>СберАвто, Team63Auto</t>
-        </is>
-      </c>
-      <c r="D65" s="4" t="inlineStr"/>
-      <c r="E65" s="7" t="inlineStr">
-        <is>
-          <t>РФ</t>
-        </is>
-      </c>
-      <c r="F65" s="7" t="inlineStr">
-        <is>
-          <t>HYUNDAI, CHERY &amp; TENET</t>
-        </is>
-      </c>
-      <c r="G65" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H65" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I65" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J65" s="7" t="inlineStr">
-        <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+      <c r="B65" s="17" t="inlineStr">
+        <is>
+          <t>ГК Автомир</t>
+        </is>
+      </c>
+      <c r="C65" s="17" t="inlineStr">
+        <is>
+          <t>ГК АВТОМИР</t>
+        </is>
+      </c>
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>7730569353</t>
+        </is>
+      </c>
+      <c r="E65" s="17" t="inlineStr">
+        <is>
+          <t>Москва</t>
+        </is>
+      </c>
+      <c r="F65" s="17" t="inlineStr">
+        <is>
+          <t>SOLARIS</t>
+        </is>
+      </c>
+      <c r="G65" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="H65" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="J65" s="17" t="inlineStr">
+        <is>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -3526,27 +3526,27 @@
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>Tenet Центр Ника Авто</t>
+          <t>Fresh Haval мин воды</t>
         </is>
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>Tenet Центр Ника Авто</t>
+          <t>Fresh Haval мин воды</t>
         </is>
       </c>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>5638074027</t>
+          <t>3443137377</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
         <is>
-          <t>Орск</t>
+          <t>Минеральные Воды</t>
         </is>
       </c>
       <c r="F66" s="11" t="inlineStr">
         <is>
-          <t>CHERY</t>
+          <t>HAVAL</t>
         </is>
       </c>
       <c r="G66" s="10" t="n">
@@ -3570,27 +3570,27 @@
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>ГК Арконт</t>
+          <t>Fresh Haval Ростов</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>ГК Арконт</t>
+          <t>Fresh Haval Ростов</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>3443113810</t>
+          <t>3443137377</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>Волгоград</t>
+          <t>Ростов-на-Дону</t>
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>HAVAL</t>
         </is>
       </c>
       <c r="G67" s="6" t="n">
@@ -3614,27 +3614,23 @@
       </c>
       <c r="B68" s="11" t="inlineStr">
         <is>
-          <t>ТВС Моторс</t>
+          <t>Team63Auto</t>
         </is>
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>ТВС Моторс</t>
-        </is>
-      </c>
-      <c r="D68" s="8" t="inlineStr">
-        <is>
-          <t>5610215334</t>
-        </is>
-      </c>
+          <t>СберАвто, Team63Auto</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr"/>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>Оренбург</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F68" s="11" t="inlineStr">
         <is>
-          <t>CHERY</t>
+          <t>CHERY &amp; TENET, HYUNDAI</t>
         </is>
       </c>
       <c r="G68" s="10" t="n">
@@ -3648,7 +3644,7 @@
       </c>
       <c r="J68" s="11" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -3658,22 +3654,22 @@
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>Фрэш Авто</t>
+          <t>Tenet Центр Ника Авто</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Фрэш Авто</t>
+          <t>Tenet Центр Ника Авто</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>7724423589</t>
+          <t>5638074027</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>Воронеж</t>
+          <t>Орск</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
@@ -3702,27 +3698,27 @@
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>Чери Центр Автофорум</t>
+          <t>ГК Арконт</t>
         </is>
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>Чери Центр Автофорум</t>
+          <t>ГК Арконт</t>
         </is>
       </c>
       <c r="D70" s="8" t="inlineStr">
         <is>
-          <t>6452947574</t>
+          <t>3443113810</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>Саратов</t>
+          <t>Волгоград</t>
         </is>
       </c>
       <c r="F70" s="11" t="inlineStr">
         <is>
-          <t>CHERY</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G70" s="10" t="n">
@@ -3746,22 +3742,22 @@
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>ЧЕРИ ЦЕНТР АГАТ-АВТО Онлайн Иркутск</t>
+          <t>ТВС Моторс</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>ЧЕРИ ЦЕНТР АГАТ-АВТО Онлайн Иркутск</t>
+          <t>ТВС Моторс</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>3804048079</t>
+          <t>5610215334</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>Иркутск</t>
+          <t>Оренбург</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr">
@@ -3790,22 +3786,22 @@
       </c>
       <c r="B72" s="11" t="inlineStr">
         <is>
-          <t>ЧЕРИ ЦЕНТР НИЖЕГОРОДЕЦ ОНЛАЙН</t>
+          <t>Фрэш Авто</t>
         </is>
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>ЧЕРИ ЦЕНТР НИЖЕГОРОДЕЦ ОНЛАЙН</t>
+          <t>Фрэш Авто</t>
         </is>
       </c>
       <c r="D72" s="8" t="inlineStr">
         <is>
-          <t>5257164835</t>
+          <t>7724423589</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>Нижний Новгород</t>
+          <t>Воронеж</t>
         </is>
       </c>
       <c r="F72" s="11" t="inlineStr">
@@ -3834,75 +3830,207 @@
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
+          <t>Чери Центр Автофорум</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Чери Центр Автофорум</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>6452947574</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>Саратов</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>CHERY</t>
+        </is>
+      </c>
+      <c r="G73" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" s="7" t="inlineStr">
+        <is>
+          <t>OEM СберАвто финал (15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="B74" s="11" t="inlineStr">
+        <is>
+          <t>ЧЕРИ ЦЕНТР АГАТ-АВТО Онлайн Иркутск</t>
+        </is>
+      </c>
+      <c r="C74" s="11" t="inlineStr">
+        <is>
+          <t>ЧЕРИ ЦЕНТР АГАТ-АВТО Онлайн Иркутск</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>3804048079</t>
+        </is>
+      </c>
+      <c r="E74" s="11" t="inlineStr">
+        <is>
+          <t>Иркутск</t>
+        </is>
+      </c>
+      <c r="F74" s="11" t="inlineStr">
+        <is>
+          <t>CHERY</t>
+        </is>
+      </c>
+      <c r="G74" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" s="11" t="inlineStr">
+        <is>
+          <t>OEM СберАвто финал (15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="4" t="n">
+        <v>71</v>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>ЧЕРИ ЦЕНТР НИЖЕГОРОДЕЦ ОНЛАЙН</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>ЧЕРИ ЦЕНТР НИЖЕГОРОДЕЦ ОНЛАЙН</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>5257164835</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>Нижний Новгород</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="inlineStr">
+        <is>
+          <t>CHERY</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" s="7" t="inlineStr">
+        <is>
+          <t>OEM СберАвто финал (15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="20" customHeight="1">
+      <c r="A76" s="8" t="n">
+        <v>72</v>
+      </c>
+      <c r="B76" s="11" t="inlineStr">
+        <is>
           <t>ЧЕРИ ЦЕНТР ПЛАНЕТА АВТО ВОСТОК</t>
         </is>
       </c>
-      <c r="C73" s="7" t="inlineStr">
+      <c r="C76" s="11" t="inlineStr">
         <is>
           <t>ЧЕРИ ЦЕНТР ПЛАНЕТА АВТО ВОСТОК</t>
         </is>
       </c>
-      <c r="D73" s="4" t="inlineStr">
+      <c r="D76" s="8" t="inlineStr">
         <is>
           <t>7447124619</t>
         </is>
       </c>
-      <c r="E73" s="7" t="inlineStr">
+      <c r="E76" s="11" t="inlineStr">
         <is>
           <t>Челябинск</t>
         </is>
       </c>
-      <c r="F73" s="7" t="inlineStr">
+      <c r="F76" s="11" t="inlineStr">
         <is>
           <t>CHERY</t>
         </is>
       </c>
-      <c r="G73" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H73" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I73" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J73" s="7" t="inlineStr">
-        <is>
-          <t>OEM СберАвто финал (15)</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="24" customHeight="1">
-      <c r="A74" s="12" t="inlineStr"/>
-      <c r="B74" s="13" t="inlineStr">
+      <c r="G76" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I76" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" s="11" t="inlineStr">
+        <is>
+          <t>OEM СберАвто финал (15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="24" customHeight="1">
+      <c r="A77" s="12" t="inlineStr"/>
+      <c r="B77" s="13" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="C74" s="13" t="inlineStr">
-        <is>
-          <t>69 объектов</t>
-        </is>
-      </c>
-      <c r="D74" s="12" t="n"/>
-      <c r="E74" s="12" t="n"/>
-      <c r="F74" s="12" t="n"/>
-      <c r="G74" s="14">
-        <f>SUM(G5:G73)</f>
+      <c r="C77" s="13" t="inlineStr">
+        <is>
+          <t>72 объектов</t>
+        </is>
+      </c>
+      <c r="D77" s="12" t="n"/>
+      <c r="E77" s="12" t="n"/>
+      <c r="F77" s="12" t="n"/>
+      <c r="G77" s="14">
+        <f>SUM(G5:G76)</f>
         <v/>
       </c>
-      <c r="H74" s="14">
-        <f>SUM(H5:H73)</f>
+      <c r="H77" s="14">
+        <f>SUM(H5:H76)</f>
         <v/>
       </c>
-      <c r="I74" s="14">
-        <f>SUM(I5:I73)</f>
+      <c r="I77" s="14">
+        <f>SUM(I5:I76)</f>
         <v/>
       </c>
-      <c r="J74" s="12" t="n"/>
+      <c r="J77" s="12" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J73"/>
+  <autoFilter ref="A4:J76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3921,7 +4049,7 @@
     <col width="65" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
@@ -6785,7 +6913,7 @@
       </c>
       <c r="F68" s="17" t="inlineStr">
         <is>
-          <t>Geely, Belgee, JETOUR</t>
+          <t>JETOUR, Belgee, Geely</t>
         </is>
       </c>
       <c r="G68" s="18" t="n">
@@ -6825,7 +6953,7 @@
       </c>
       <c r="F69" s="17" t="inlineStr">
         <is>
-          <t>LADA, GAC, HAVAL</t>
+          <t>LADA, HAVAL, GAC</t>
         </is>
       </c>
       <c r="G69" s="18" t="n">
@@ -7514,7 +7642,7 @@
       </c>
       <c r="C85" s="17" t="inlineStr">
         <is>
-          <t>ООО "МЛАДА - АВТО" online, ГК Техцентр Гранд</t>
+          <t>ГК Техцентр Гранд, ООО "МЛАДА - АВТО" online</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr"/>
@@ -7525,7 +7653,7 @@
       </c>
       <c r="F85" s="17" t="inlineStr">
         <is>
-          <t>SOUEAST, JETOUR</t>
+          <t>JETOUR, SOUEAST</t>
         </is>
       </c>
       <c r="G85" s="18" t="n">
@@ -9185,7 +9313,7 @@
       </c>
       <c r="F123" s="17" t="inlineStr">
         <is>
-          <t>SOUEAST, JETOUR</t>
+          <t>JETOUR, SOUEAST</t>
         </is>
       </c>
       <c r="G123" s="18" t="n">
@@ -10610,7 +10738,7 @@
       </c>
       <c r="C156" s="17" t="inlineStr">
         <is>
-          <t>ONLINE ФДЦ АВТО-МОТОРС Сургут, Online ООО АВТО-МОТОРС Лада</t>
+          <t>Online ООО АВТО-МОТОРС Лада, ONLINE ФДЦ АВТО-МОТОРС Сургут</t>
         </is>
       </c>
       <c r="D156" s="16" t="inlineStr"/>
@@ -10661,7 +10789,7 @@
       </c>
       <c r="F157" s="7" t="inlineStr">
         <is>
-          <t>JETOUR, RENAULT, EXEED</t>
+          <t>RENAULT, JETOUR, Belgee</t>
         </is>
       </c>
       <c r="G157" s="6" t="n">
@@ -12661,7 +12789,7 @@
       </c>
       <c r="F203" s="7" t="inlineStr">
         <is>
-          <t>LAND, RENAULT, TOYOTA</t>
+          <t>RENAULT, TOYOTA, LAND</t>
         </is>
       </c>
       <c r="G203" s="6" t="n">
@@ -13292,37 +13420,37 @@
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>ФДЦ Автосеть АМК РФ</t>
-        </is>
-      </c>
-      <c r="C5" s="17" t="inlineStr"/>
-      <c r="D5" s="16" t="inlineStr">
-        <is>
-          <t>0245968960</t>
-        </is>
-      </c>
+          <t>ГК Арконт</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>Online ООО "АРКОНТ В"</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr"/>
       <c r="E5" s="17" t="inlineStr">
         <is>
-          <t>Уфа</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
-          <t>CHERY</t>
+          <t>JETOUR, SOUEAST</t>
         </is>
       </c>
       <c r="G5" s="18" t="n">
-        <v>61</v>
+        <v>11</v>
       </c>
       <c r="H5" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I5" s="18" t="n">
-        <v>61</v>
+        <v>11</v>
       </c>
       <c r="J5" s="17" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -13332,37 +13460,41 @@
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>ГК Арконт</t>
+          <t>Башавтоком / Чанган Центр</t>
         </is>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
-          <t>Online ООО "АРКОНТ В"</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr"/>
+          <t>Башавтоком</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>0278105341</t>
+        </is>
+      </c>
       <c r="E6" s="17" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Стерлитамак</t>
         </is>
       </c>
       <c r="F6" s="17" t="inlineStr">
         <is>
-          <t>SOUEAST, JETOUR</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G6" s="18" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H6" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I6" s="18" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="J6" s="17" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -13431,7 +13563,7 @@
       </c>
       <c r="E8" s="17" t="inlineStr">
         <is>
-          <t>Стерлитамак</t>
+          <t>Уфа</t>
         </is>
       </c>
       <c r="F8" s="17" t="inlineStr">
@@ -13470,7 +13602,7 @@
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
-          <t>0278105341</t>
+          <t>0277063113</t>
         </is>
       </c>
       <c r="E9" s="17" t="inlineStr">
@@ -13480,7 +13612,7 @@
       </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>CHANGAN</t>
         </is>
       </c>
       <c r="G9" s="18" t="n">
@@ -13524,7 +13656,7 @@
       </c>
       <c r="F10" s="17" t="inlineStr">
         <is>
-          <t>CHANGAN</t>
+          <t>DEEPAL</t>
         </is>
       </c>
       <c r="G10" s="18" t="n">
@@ -13548,37 +13680,37 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>Башавтоком / Чанган Центр</t>
+          <t>ТСАЦ Июль</t>
         </is>
       </c>
       <c r="C11" s="17" t="inlineStr">
         <is>
-          <t>Башавтоком</t>
+          <t>Июль</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>0277063113</t>
+          <t>7449109091</t>
         </is>
       </c>
       <c r="E11" s="17" t="inlineStr">
         <is>
-          <t>Уфа</t>
+          <t>Екатеринбург</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
-          <t>DEEPAL</t>
+          <t>CHERY</t>
         </is>
       </c>
       <c r="G11" s="18" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="H11" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="18" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J11" s="17" t="inlineStr">
         <is>
@@ -13612,7 +13744,7 @@
       </c>
       <c r="F12" s="17" t="inlineStr">
         <is>
-          <t>CHERY</t>
+          <t>OMODA</t>
         </is>
       </c>
       <c r="G12" s="18" t="n">
@@ -13641,12 +13773,12 @@
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>Июль</t>
+          <t>ТСАЦ Июль</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>7449109091</t>
+          <t>6670086484</t>
         </is>
       </c>
       <c r="E13" s="17" t="inlineStr">
@@ -13656,7 +13788,7 @@
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
-          <t>OMODA</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G13" s="18" t="n">
@@ -13680,27 +13812,27 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>ТСАЦ Июль</t>
+          <t>Форвард</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>ТСАЦ Июль</t>
+          <t>Форвард Авто</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>6670086484</t>
+          <t>0276945049</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
         <is>
-          <t>Екатеринбург</t>
+          <t>Уфа</t>
         </is>
       </c>
       <c r="F14" s="17" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>CHERY</t>
         </is>
       </c>
       <c r="G14" s="18" t="n">
@@ -13734,17 +13866,17 @@
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>0276945049</t>
+          <t>5902174928</t>
         </is>
       </c>
       <c r="E15" s="17" t="inlineStr">
         <is>
-          <t>Уфа</t>
+          <t>Ижевск</t>
         </is>
       </c>
       <c r="F15" s="17" t="inlineStr">
         <is>
-          <t>CHERY</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G15" s="18" t="n">
@@ -13768,37 +13900,37 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>Форвард</t>
+          <t>ГК Артан</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>Форвард Авто</t>
+          <t>ГК Артан</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>5902174928</t>
+          <t>5262004523</t>
         </is>
       </c>
       <c r="E16" s="17" t="inlineStr">
         <is>
-          <t>Ижевск</t>
+          <t>Нижний Новгород</t>
         </is>
       </c>
       <c r="F16" s="17" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G16" s="18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H16" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I16" s="18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J16" s="17" t="inlineStr">
         <is>
@@ -13812,27 +13944,27 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>ГК Артан</t>
+          <t>Нижегородец</t>
         </is>
       </c>
       <c r="C17" s="17" t="inlineStr">
         <is>
-          <t>ГК Артан</t>
+          <t>Нижегородец</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>5262004523</t>
+          <t>5257164835</t>
         </is>
       </c>
       <c r="E17" s="17" t="inlineStr">
         <is>
-          <t>Нижний Новгород</t>
+          <t>Арзамас</t>
         </is>
       </c>
       <c r="F17" s="17" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>CHERY</t>
         </is>
       </c>
       <c r="G17" s="18" t="n">
@@ -13871,7 +14003,7 @@
       </c>
       <c r="E18" s="17" t="inlineStr">
         <is>
-          <t>Арзамас</t>
+          <t>Москва</t>
         </is>
       </c>
       <c r="F18" s="17" t="inlineStr">
@@ -13900,22 +14032,18 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>Нижегородец</t>
-        </is>
-      </c>
-      <c r="C19" s="17" t="inlineStr">
-        <is>
-          <t>Нижегородец</t>
-        </is>
-      </c>
+          <t>ООО "ТД АРМАДА-АВТО</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr"/>
       <c r="D19" s="16" t="inlineStr">
         <is>
-          <t>5257164835</t>
+          <t>0245968960</t>
         </is>
       </c>
       <c r="E19" s="17" t="inlineStr">
         <is>
-          <t>Москва</t>
+          <t>Уфа</t>
         </is>
       </c>
       <c r="F19" s="17" t="inlineStr">
@@ -13944,37 +14072,41 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>ООО "ТД АРМАДА-АВТО</t>
+          <t>Эксперт Авто (Самара)</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>ONLINE ООО "ТД АРМАДА-АВТО"</t>
-        </is>
-      </c>
-      <c r="D20" s="16" t="inlineStr"/>
+          <t>Эксперт Авто</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>6312147970</t>
+        </is>
+      </c>
       <c r="E20" s="17" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Самара</t>
         </is>
       </c>
       <c r="F20" s="17" t="inlineStr">
         <is>
-          <t>SOUEAST, JETOUR</t>
+          <t>GEELY,BELGEE,KNEWSTAR</t>
         </is>
       </c>
       <c r="G20" s="18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H20" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I20" s="18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J20" s="17" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -13989,12 +14121,12 @@
       </c>
       <c r="C21" s="17" t="inlineStr">
         <is>
-          <t>Эксперт Авто</t>
+          <t>ЭКСПЕРТ АВТО</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr">
         <is>
-          <t>6312147970</t>
+          <t>6314034107</t>
         </is>
       </c>
       <c r="E21" s="17" t="inlineStr">
@@ -14004,7 +14136,7 @@
       </c>
       <c r="F21" s="17" t="inlineStr">
         <is>
-          <t>GEELY,BELGEE,KNEWSTAR</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G21" s="18" t="n">
@@ -14033,12 +14165,12 @@
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>ЭКСПЕРТ АВТО</t>
+          <t>Эксперт Авто</t>
         </is>
       </c>
       <c r="D22" s="16" t="inlineStr">
         <is>
-          <t>6314034107</t>
+          <t>6312147970</t>
         </is>
       </c>
       <c r="E22" s="17" t="inlineStr">
@@ -14048,7 +14180,7 @@
       </c>
       <c r="F22" s="17" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>SOLARIS</t>
         </is>
       </c>
       <c r="G22" s="18" t="n">
@@ -14072,41 +14204,37 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>Эксперт Авто (Самара)</t>
+          <t>ГК БН-Моторс</t>
         </is>
       </c>
       <c r="C23" s="17" t="inlineStr">
         <is>
-          <t>Эксперт Авто</t>
-        </is>
-      </c>
-      <c r="D23" s="16" t="inlineStr">
-        <is>
-          <t>6312147970</t>
-        </is>
-      </c>
+          <t>ГК БН-МОТОРС, БНМ, ООО "МБ-БРЯНСК" ONLINE</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr"/>
       <c r="E23" s="17" t="inlineStr">
         <is>
-          <t>Самара</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F23" s="17" t="inlineStr">
         <is>
-          <t>SOLARIS</t>
+          <t>LADA, JETOUR, SOUEAST</t>
         </is>
       </c>
       <c r="G23" s="18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H23" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I23" s="18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J23" s="17" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -14116,12 +14244,12 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>ГК БН-Моторс</t>
+          <t>ГК Сильвер</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>ГК БН-МОТОРС, БНМ, ООО "МБ-БРЯНСК" ONLINE</t>
+          <t>ООО "СИЛЬВЕР-АВТО ПЛЮС" ONLINE</t>
         </is>
       </c>
       <c r="D24" s="16" t="inlineStr"/>
@@ -14132,7 +14260,7 @@
       </c>
       <c r="F24" s="17" t="inlineStr">
         <is>
-          <t>LADA, SOUEAST, JETOUR</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G24" s="18" t="n">
@@ -14156,12 +14284,12 @@
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>ГК Сильвер</t>
+          <t>ООО "ВОСТОК МОТОРС</t>
         </is>
       </c>
       <c r="C25" s="17" t="inlineStr">
         <is>
-          <t>ООО "СИЛЬВЕР-АВТО ПЛЮС" ONLINE</t>
+          <t>ООО "ВОСТОК МОТОРС" ONLINE</t>
         </is>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
@@ -14196,18 +14324,22 @@
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>ООО "ВОСТОК МОТОРС</t>
+          <t>JETOUR АвтоПремьер Зубово</t>
         </is>
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>ООО "ВОСТОК МОТОРС" ONLINE</t>
-        </is>
-      </c>
-      <c r="D26" s="16" t="inlineStr"/>
+          <t>JETOUR АвтоПремьер Зубово</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>0245961925</t>
+        </is>
+      </c>
       <c r="E26" s="17" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Уфа</t>
         </is>
       </c>
       <c r="F26" s="17" t="inlineStr">
@@ -14216,17 +14348,17 @@
         </is>
       </c>
       <c r="G26" s="18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H26" s="18" t="n">
         <v>0</v>
       </c>
       <c r="I26" s="18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J26" s="17" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -14236,27 +14368,23 @@
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>JETOUR АвтоПремьер Зубово</t>
+          <t>Автохолдинг Максимум</t>
         </is>
       </c>
       <c r="C27" s="17" t="inlineStr">
         <is>
-          <t>JETOUR АвтоПремьер Зубово</t>
-        </is>
-      </c>
-      <c r="D27" s="16" t="inlineStr">
-        <is>
-          <t>0245961925</t>
-        </is>
-      </c>
+          <t>ЗАО "АВТОХОЛДИНГ" LUCKY MOTORS ONLINE</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr"/>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>Уфа</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F27" s="17" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>JETOUR, SOUEAST</t>
         </is>
       </c>
       <c r="G27" s="18" t="n">
@@ -14270,7 +14398,7 @@
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -14280,12 +14408,12 @@
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>Автохолдинг Максимум</t>
+          <t>ГК АГАТ</t>
         </is>
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>ЗАО "АВТОХОЛДИНГ" LUCKY MOTORS ONLINE</t>
+          <t>ONLINE АГАТ CHERY/O&amp;J (ООО "АВТО-КОНТИНЕНТ")</t>
         </is>
       </c>
       <c r="D28" s="16" t="inlineStr"/>
@@ -14296,7 +14424,7 @@
       </c>
       <c r="F28" s="17" t="inlineStr">
         <is>
-          <t>SOUEAST, JETOUR</t>
+          <t>OMODA &amp; JAECOO, CHERY &amp; TENET</t>
         </is>
       </c>
       <c r="G28" s="18" t="n">
@@ -14320,23 +14448,27 @@
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>ГК АГАТ</t>
+          <t>Дав-Авто</t>
         </is>
       </c>
       <c r="C29" s="17" t="inlineStr">
         <is>
-          <t>ONLINE АГАТ CHERY/O&amp;J (ООО "АВТО-КОНТИНЕНТ")</t>
-        </is>
-      </c>
-      <c r="D29" s="16" t="inlineStr"/>
+          <t>Дав-Авто</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>5904329165</t>
+        </is>
+      </c>
       <c r="E29" s="17" t="inlineStr">
         <is>
-          <t>РФ</t>
+          <t>Пермь</t>
         </is>
       </c>
       <c r="F29" s="17" t="inlineStr">
         <is>
-          <t>CHERY &amp; TENET, OMODA &amp; JAECOO</t>
+          <t>CHANGAN</t>
         </is>
       </c>
       <c r="G29" s="18" t="n">
@@ -14350,7 +14482,7 @@
       </c>
       <c r="J29" s="17" t="inlineStr">
         <is>
-          <t>Сделки Сентябрь 2026 (Битрикс)</t>
+          <t>OEM СберАвто финал (15)</t>
         </is>
       </c>
     </row>
@@ -14380,7 +14512,7 @@
       </c>
       <c r="F30" s="17" t="inlineStr">
         <is>
-          <t>CHANGAN</t>
+          <t>DEEPAL</t>
         </is>
       </c>
       <c r="G30" s="18" t="n">
@@ -14404,27 +14536,27 @@
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>Дав-Авто</t>
+          <t>Никко</t>
         </is>
       </c>
       <c r="C31" s="17" t="inlineStr">
         <is>
-          <t>Дав-Авто</t>
+          <t>Никко</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
-          <t>5904329165</t>
+          <t>5638061236</t>
         </is>
       </c>
       <c r="E31" s="17" t="inlineStr">
         <is>
-          <t>Пермь</t>
+          <t>Оренбург</t>
         </is>
       </c>
       <c r="F31" s="17" t="inlineStr">
         <is>
-          <t>DEEPAL</t>
+          <t>JETOUR</t>
         </is>
       </c>
       <c r="G31" s="18" t="n">
@@ -14448,27 +14580,23 @@
       </c>
       <c r="B32" s="17" t="inlineStr">
         <is>
-          <t>Никко</t>
+          <t>Олимп (Кубань)</t>
         </is>
       </c>
       <c r="C32" s="17" t="inlineStr">
         <is>
-          <t>Никко</t>
-        </is>
-      </c>
-      <c r="D32" s="16" t="inlineStr">
-        <is>
-          <t>5638061236</t>
-        </is>
-      </c>
+          <t>ONLINE Олимп, ONLINE Олимп (ООО "ТЕМП АВТО КУБАНЬ")</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr"/>
       <c r="E32" s="17" t="inlineStr">
         <is>
-          <t>Оренбург</t>
+          <t>РФ</t>
         </is>
       </c>
       <c r="F32" s="17" t="inlineStr">
         <is>
-          <t>JETOUR</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G32" s="18" t="n">
@@ -14482,7 +14610,7 @@
       </c>
       <c r="J32" s="17" t="inlineStr">
         <is>
-          <t>OEM СберАвто финал (15)</t>
+          <t>Сделки Сентябрь 2026 (Битрикс)</t>
         </is>
       </c>
     </row>
@@ -14492,12 +14620,12 @@
       </c>
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>Олимп (Кубань)</t>
+          <t>Приоритет_Автобан</t>
         </is>
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
-          <t>ONLINE Олимп (ООО "ТЕМП АВТО КУБАНЬ"), ONLINE Олимп</t>
+          <t>Приоритет_Автобан, ONLINE ООО "АВТОБАН-ВОСТОК"</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr"/>
@@ -14508,7 +14636,7 @@
       </c>
       <c r="F33" s="17" t="inlineStr">
         <is>
-          <t>LADA</t>
+          <t>JETOUR, SKODA, SOUEAST</t>
         </is>
       </c>
       <c r="G33" s="18" t="n">
@@ -14532,12 +14660,12 @@
       </c>
       <c r="B34" s="17" t="inlineStr">
         <is>
-          <t>Приоритет_Автобан</t>
+          <t>ТВС Моторс</t>
         </is>
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>Приоритет_Автобан, ONLINE ООО "АВТОБАН-ВОСТОК"</t>
+          <t>ONLINE CHERY ТВС Моторс (ООО "ЗОЛОТОЙ ДРАКОН")</t>
         </is>
       </c>
       <c r="D34" s="16" t="inlineStr"/>
@@ -14548,7 +14676,7 @@
       </c>
       <c r="F34" s="17" t="inlineStr">
         <is>
-          <t>SKODA, SOUEAST, JETOUR</t>
+          <t>CHERY &amp; TENET</t>
         </is>
       </c>
       <c r="G34" s="18" t="n">
@@ -14572,12 +14700,12 @@
       </c>
       <c r="B35" s="17" t="inlineStr">
         <is>
-          <t>ТВС Моторс</t>
+          <t>ФДЦ Автосеть АМК РФ</t>
         </is>
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
-          <t>ONLINE CHERY ТВС Моторс (ООО "ЗОЛОТОЙ ДРАКОН")</t>
+          <t>ONLINE АМК Тольятти (ООО "АМ Компани"), ONLINE АМК Самара ООО "УРАЛ-ЛАДА"</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr"/>
@@ -14588,7 +14716,7 @@
       </c>
       <c r="F35" s="17" t="inlineStr">
         <is>
-          <t>CHERY &amp; TENET</t>
+          <t>LADA</t>
         </is>
       </c>
       <c r="G35" s="18" t="n">
@@ -15257,7 +15385,7 @@
       </c>
       <c r="C51" s="17" t="inlineStr">
         <is>
-          <t>ONLINE Самара-Лада, Самара-Лада (ООО Самара-Лада)/ Продажи МегаМаркета + Online</t>
+          <t>Самара-Лада (ООО Самара-Лада)/ Продажи МегаМаркета + Online, ONLINE Самара-Лада</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr"/>
@@ -15425,7 +15553,7 @@
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>СберАвто, Нижегородец</t>
+          <t>Нижегородец, СберАвто</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr"/>
@@ -17472,7 +17600,7 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="41" customWidth="1" min="2" max="2"/>
-    <col width="91" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -18480,7 +18608,7 @@
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>ООО "ДИНАМИКА ЧЕРЕПОВЕЦ" ONLINE, СберАвто</t>
+          <t>ООО "ДИНАМИКА АРХАНГЕЛЬСК" ONLINE, СберАвто</t>
         </is>
       </c>
       <c r="D26" s="16" t="inlineStr"/>
@@ -19476,7 +19604,7 @@
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>ONLINE Прагматика (ООО Прагматика Мурманск), ONLINE Пилот ФДЦ Прагматика СпБ В-НГРД ПСКВ</t>
+          <t>Атик, ONLINE Пилот ФДЦ Прагматика СпБ В-НГРД ПСКВ</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr"/>
@@ -20307,7 +20435,7 @@
       </c>
       <c r="F68" s="11" t="inlineStr">
         <is>
-          <t>Geely, HAVAL</t>
+          <t>HAVAL, Geely</t>
         </is>
       </c>
       <c r="G68" s="10" t="n">
@@ -22978,7 +23106,7 @@
     <col width="35" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="33" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
@@ -28651,7 +28779,7 @@
       </c>
       <c r="C132" s="17" t="inlineStr">
         <is>
-          <t>СберАвто, ONLINE ООО "АВТОСФЕРА"</t>
+          <t>ONLINE ООО "АВТОСФЕРА", СберАвто</t>
         </is>
       </c>
       <c r="D132" s="16" t="inlineStr"/>
@@ -28662,7 +28790,7 @@
       </c>
       <c r="F132" s="17" t="inlineStr">
         <is>
-          <t>JELAND, SOUEAST, CHERY &amp; TENET</t>
+          <t>CHERY &amp; TENET, JETOUR, JELAND</t>
         </is>
       </c>
       <c r="G132" s="18" t="n">

</xml_diff>